<commit_message>
Code after Portugal New Hire Completed
</commit_message>
<xml_diff>
--- a/Data/Hires/Workday_NewHire_Czechia_Regression_PK14.xlsx
+++ b/Data/Hires/Workday_NewHire_Czechia_Regression_PK14.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{B7A08F11-A613-4D61-ABD9-FE3D584268FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{F4FCC049-59D5-4472-9686-D26CD4CF0BF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1068" yWindow="-108" windowWidth="22080" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1000" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="242">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -259,7 +259,7 @@
     <t>Test1</t>
   </si>
   <si>
-    <t>10697638</t>
+    <t>10697730</t>
   </si>
   <si>
     <t>Passed</t>
@@ -274,7 +274,7 @@
     <t>CzOne</t>
   </si>
   <si>
-    <t>TwentyFiveMarchTwentyFive</t>
+    <t>TwentyFiveAprilSeven</t>
   </si>
   <si>
     <t>770 272 784</t>
@@ -412,7 +412,7 @@
     <t>Test2</t>
   </si>
   <si>
-    <t>10697639</t>
+    <t>10697766</t>
   </si>
   <si>
     <t>895 Store Management (Jaziz Wezupa (10573442))</t>
@@ -421,7 +421,7 @@
     <t>CzTwo</t>
   </si>
   <si>
-    <t>Auto 26672617</t>
+    <t>Auto 25154444</t>
   </si>
   <si>
     <t>Department Manager_NEW</t>
@@ -442,7 +442,7 @@
     <t>Test3</t>
   </si>
   <si>
-    <t>10697640</t>
+    <t>10697731</t>
   </si>
   <si>
     <t>CzThree</t>
@@ -478,13 +478,10 @@
     <t>Test4</t>
   </si>
   <si>
-    <t>10697641</t>
-  </si>
-  <si>
     <t>CzFour</t>
   </si>
   <si>
-    <t>Auto 79872584</t>
+    <t>Auto 9592202</t>
   </si>
   <si>
     <t>Assistant Store Manager_NEW</t>
@@ -508,7 +505,7 @@
     <t>Test5</t>
   </si>
   <si>
-    <t>Test failed for 'CzFive TwentyFiveMarchTwentyFive' Employee: Errors and AlertsErrorPage Error- You have not entered an amount within the Compensation Guidelines.     (Employee Compensation Event For Hire Employee)AlertPage Alert- "Warning: You have entered an amount that is outside of the range or more than 10% higher than the current salary.  Please re-enter an amount inside the range, below 10% or continue and it will be sent for approval."     (Employee Compensation Event For Hire Employee) &amp; find failed Screenshot Path:-&gt;H:\WorkdayPlaywright/WorkdayFailedScreenshot/2025-03-25T13-56-11-535Z.png</t>
+    <t>Test failed for 'CzFive TwentyFiveAprilSeven' Employee: Errors and AlertsErrorPage Error- You have not entered an amount within the Compensation Guidelines.     (Employee Compensation Event For Hire Employee)AlertPage Alert- "Warning: You have entered an amount that is outside of the range or more than 10% higher than the current salary.  Please re-enter an amount inside the range, below 10% or continue and it will be sent for approval."     (Employee Compensation Event For Hire Employee) &amp; find failed Screenshot Path:-&gt;H:\WorkdayPlaywright/WorkdayFailedScreenshot/2025-04-07T05-12-02-845Z.png</t>
   </si>
   <si>
     <t>Failed</t>
@@ -544,19 +541,13 @@
     <t>Test6</t>
   </si>
   <si>
-    <t>10697655</t>
-  </si>
-  <si>
     <t>CzSix</t>
   </si>
   <si>
-    <t>TwentyFiveMarchTwentyFiveB</t>
-  </si>
-  <si>
     <t>771 272 784</t>
   </si>
   <si>
-    <t>Auto 13348423</t>
+    <t>Auto 39660385</t>
   </si>
   <si>
     <t>In-Store Visual Merchandising Manager_NEW</t>
@@ -580,12 +571,12 @@
     <t>Test7</t>
   </si>
   <si>
+    <t>10697733</t>
+  </si>
+  <si>
     <t>CzSeven</t>
   </si>
   <si>
-    <t>TwentyFiveMarchTwentyFiveA</t>
-  </si>
-  <si>
     <t>772 272 784</t>
   </si>
   <si>
@@ -604,16 +595,13 @@
     <t>Test8</t>
   </si>
   <si>
-    <t>10697643</t>
-  </si>
-  <si>
     <t>CzEight</t>
   </si>
   <si>
     <t>773 272 784</t>
   </si>
   <si>
-    <t>Auto 16094310</t>
+    <t>Auto 79587467</t>
   </si>
   <si>
     <t>Store Manager_NEW</t>
@@ -628,7 +616,7 @@
     <t>Test9</t>
   </si>
   <si>
-    <t>10697644</t>
+    <t>10697735</t>
   </si>
   <si>
     <t>CzNine</t>
@@ -649,16 +637,13 @@
     <t>Test10</t>
   </si>
   <si>
-    <t>10697646</t>
-  </si>
-  <si>
     <t>CzTen</t>
   </si>
   <si>
     <t>775 272 784</t>
   </si>
   <si>
-    <t>Auto 11194568</t>
+    <t>Auto 62280742</t>
   </si>
   <si>
     <t>Team Manager - Retail_NEW</t>
@@ -673,7 +658,7 @@
     <t>Test11</t>
   </si>
   <si>
-    <t>10697647</t>
+    <t>10697737</t>
   </si>
   <si>
     <t>CzEleven</t>
@@ -697,16 +682,13 @@
     <t>Test12</t>
   </si>
   <si>
-    <t>10697649</t>
-  </si>
-  <si>
     <t>CzTweve</t>
   </si>
   <si>
     <t>777 272 784</t>
   </si>
   <si>
-    <t>Auto 54400108</t>
+    <t>Auto 71162593</t>
   </si>
   <si>
     <t>In-Store P&amp;C Manager_NEW</t>
@@ -721,7 +703,7 @@
     <t>Test13</t>
   </si>
   <si>
-    <t>10697650</t>
+    <t>10697739</t>
   </si>
   <si>
     <t>CzThirteen</t>
@@ -742,7 +724,7 @@
     <t>Test14</t>
   </si>
   <si>
-    <t>10697651</t>
+    <t>10697741</t>
   </si>
   <si>
     <t>CzFourteen</t>
@@ -760,7 +742,7 @@
     <t>Test15</t>
   </si>
   <si>
-    <t>10697652</t>
+    <t>10697742</t>
   </si>
   <si>
     <t>CzFifteenA</t>
@@ -1259,7 +1241,7 @@
     <col min="4" max="4" width="46.88671875" style="1" customWidth="1"/>
     <col min="5" max="5" width="7.88671875" style="1" customWidth="1"/>
     <col min="6" max="6" width="13.88671875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="27.109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="16.77734375" style="1" customWidth="1"/>
     <col min="8" max="8" width="16.109375" style="1" customWidth="1"/>
     <col min="9" max="9" width="14.77734375" style="1" customWidth="1"/>
     <col min="10" max="10" width="6.21875" style="1" customWidth="1"/>
@@ -1730,7 +1712,7 @@
         <v>104</v>
       </c>
       <c r="AT2" s="18">
-        <v>9561116906</v>
+        <v>9561118391</v>
       </c>
       <c r="AU2" s="13" t="s">
         <v>105</v>
@@ -1745,7 +1727,7 @@
         <v>107</v>
       </c>
       <c r="AY2" s="19">
-        <v>143372867</v>
+        <v>142982899</v>
       </c>
       <c r="AZ2" s="13" t="s">
         <v>105</v>
@@ -1836,7 +1818,7 @@
       <c r="A3" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="9" t="s">
         <v>127</v>
       </c>
       <c r="C3" s="8" t="s">
@@ -1974,7 +1956,7 @@
         <v>104</v>
       </c>
       <c r="AT3" s="18">
-        <v>9561117335</v>
+        <v>9561112374</v>
       </c>
       <c r="AU3" s="13" t="s">
         <v>105</v>
@@ -1989,7 +1971,7 @@
         <v>107</v>
       </c>
       <c r="AY3" s="19">
-        <v>143792868</v>
+        <v>142972900</v>
       </c>
       <c r="AZ3" s="13" t="s">
         <v>105</v>
@@ -2219,7 +2201,7 @@
         <v>104</v>
       </c>
       <c r="AT4" s="18">
-        <v>9561117445</v>
+        <v>9561115564</v>
       </c>
       <c r="AU4" s="13" t="s">
         <v>105</v>
@@ -2234,7 +2216,7 @@
         <v>107</v>
       </c>
       <c r="AY4" s="19">
-        <v>143282869</v>
+        <v>142962901</v>
       </c>
       <c r="AZ4" s="13" t="s">
         <v>105</v>
@@ -2325,8 +2307,8 @@
       <c r="A5" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="B5" s="9" t="s">
-        <v>149</v>
+      <c r="B5" s="9">
+        <v>10697732</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>77</v>
@@ -2338,7 +2320,7 @@
         <v>79</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G5" s="12" t="s">
         <v>81</v>
@@ -2399,13 +2381,13 @@
         <v>91</v>
       </c>
       <c r="Z5" s="12" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="AA5" s="8" t="s">
         <v>139</v>
       </c>
       <c r="AB5" s="8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AC5" s="8" t="s">
         <v>95</v>
@@ -2464,7 +2446,7 @@
         <v>104</v>
       </c>
       <c r="AT5" s="18">
-        <v>9561113551</v>
+        <v>9561119909</v>
       </c>
       <c r="AU5" s="13" t="s">
         <v>105</v>
@@ -2479,7 +2461,7 @@
         <v>107</v>
       </c>
       <c r="AY5" s="19">
-        <v>143272870</v>
+        <v>142952902</v>
       </c>
       <c r="AZ5" s="13" t="s">
         <v>105</v>
@@ -2518,10 +2500,10 @@
         <v>79</v>
       </c>
       <c r="BL5" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="BM5" s="14" t="s">
         <v>153</v>
-      </c>
-      <c r="BM5" s="14" t="s">
-        <v>154</v>
       </c>
       <c r="BN5" s="14" t="s">
         <v>117</v>
@@ -2539,7 +2521,7 @@
         <v>2024</v>
       </c>
       <c r="BS5" s="14" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="BT5" s="14" t="s">
         <v>120</v>
@@ -2548,10 +2530,10 @@
         <v>79</v>
       </c>
       <c r="BV5" s="20" t="s">
+        <v>155</v>
+      </c>
+      <c r="BW5" s="20" t="s">
         <v>156</v>
-      </c>
-      <c r="BW5" s="20" t="s">
-        <v>157</v>
       </c>
       <c r="BX5" s="20">
         <v>207</v>
@@ -2568,13 +2550,13 @@
     </row>
     <row r="6" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="B6" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="C6" s="8" t="s">
         <v>159</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>160</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>78</v>
@@ -2583,7 +2565,7 @@
         <v>79</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G6" s="12" t="s">
         <v>81</v>
@@ -2647,10 +2629,10 @@
         <v>92</v>
       </c>
       <c r="AA6" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="AB6" s="8" t="s">
         <v>162</v>
-      </c>
-      <c r="AB6" s="8" t="s">
-        <v>163</v>
       </c>
       <c r="AC6" s="8" t="s">
         <v>140</v>
@@ -2659,10 +2641,10 @@
         <v>96</v>
       </c>
       <c r="AE6" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="AF6" s="8" t="s">
         <v>164</v>
-      </c>
-      <c r="AF6" s="8" t="s">
-        <v>165</v>
       </c>
       <c r="AG6" s="16">
         <v>16</v>
@@ -2672,7 +2654,7 @@
         <v>45962</v>
       </c>
       <c r="AI6" s="12" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="AJ6" s="12" t="s">
         <v>101</v>
@@ -2693,7 +2675,7 @@
         <v>102</v>
       </c>
       <c r="AO6" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="AP6" s="11">
         <v>100</v>
@@ -2709,7 +2691,7 @@
         <v>104</v>
       </c>
       <c r="AT6" s="18">
-        <v>9561110493</v>
+        <v>9561112110</v>
       </c>
       <c r="AU6" s="13" t="s">
         <v>105</v>
@@ -2724,7 +2706,7 @@
         <v>107</v>
       </c>
       <c r="AY6" s="19">
-        <v>143262871</v>
+        <v>142942903</v>
       </c>
       <c r="AZ6" s="13" t="s">
         <v>105</v>
@@ -2793,10 +2775,10 @@
         <v>79</v>
       </c>
       <c r="BV6" s="20" t="s">
+        <v>167</v>
+      </c>
+      <c r="BW6" s="20" t="s">
         <v>168</v>
-      </c>
-      <c r="BW6" s="20" t="s">
-        <v>169</v>
       </c>
       <c r="BX6" s="20">
         <v>211</v>
@@ -2813,10 +2795,10 @@
     </row>
     <row r="7" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>171</v>
+        <v>169</v>
+      </c>
+      <c r="B7" s="9">
+        <v>10697765</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>77</v>
@@ -2828,13 +2810,13 @@
         <v>79</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>173</v>
+        <v>81</v>
       </c>
       <c r="H7" s="12" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="I7" s="12" t="s">
         <v>83</v>
@@ -2889,13 +2871,13 @@
         <v>91</v>
       </c>
       <c r="Z7" s="12" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="AA7" s="8" t="s">
         <v>93</v>
       </c>
       <c r="AB7" s="8" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="AC7" s="8" t="s">
         <v>140</v>
@@ -2953,7 +2935,7 @@
         <v>104</v>
       </c>
       <c r="AT7" s="18">
-        <v>9561118468</v>
+        <v>9561118017</v>
       </c>
       <c r="AU7" s="13" t="s">
         <v>105</v>
@@ -2968,7 +2950,7 @@
         <v>107</v>
       </c>
       <c r="AY7" s="19">
-        <v>143152882</v>
+        <v>142932904</v>
       </c>
       <c r="AZ7" s="13" t="s">
         <v>105</v>
@@ -3007,10 +2989,10 @@
         <v>79</v>
       </c>
       <c r="BL7" s="14" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="BM7" s="14" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="BN7" s="14" t="s">
         <v>117</v>
@@ -3028,7 +3010,7 @@
         <v>2000</v>
       </c>
       <c r="BS7" s="14" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="BT7" s="14" t="s">
         <v>120</v>
@@ -3037,10 +3019,10 @@
         <v>79</v>
       </c>
       <c r="BV7" s="20" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="BW7" s="20" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="BX7" s="20">
         <v>211</v>
@@ -3057,10 +3039,10 @@
     </row>
     <row r="8" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="B8" s="21">
-        <v>10697653</v>
+        <v>179</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>180</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>77</v>
@@ -3072,13 +3054,13 @@
         <v>79</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>184</v>
+        <v>81</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="I8" s="12" t="s">
         <v>83</v>
@@ -3139,7 +3121,7 @@
         <v>139</v>
       </c>
       <c r="AB8" s="8" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="AC8" s="8" t="s">
         <v>140</v>
@@ -3182,7 +3164,7 @@
         <v>102</v>
       </c>
       <c r="AO8" s="8" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="AP8" s="11">
         <v>100</v>
@@ -3198,7 +3180,7 @@
         <v>104</v>
       </c>
       <c r="AT8" s="18">
-        <v>9561115597</v>
+        <v>9561116499</v>
       </c>
       <c r="AU8" s="13" t="s">
         <v>105</v>
@@ -3213,7 +3195,7 @@
         <v>107</v>
       </c>
       <c r="AY8" s="19">
-        <v>143242873</v>
+        <v>142922905</v>
       </c>
       <c r="AZ8" s="13" t="s">
         <v>105</v>
@@ -3282,10 +3264,10 @@
         <v>79</v>
       </c>
       <c r="BV8" s="20" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="BW8" s="20" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="BX8" s="20">
         <v>213</v>
@@ -3302,10 +3284,10 @@
     </row>
     <row r="9" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>190</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>191</v>
+        <v>187</v>
+      </c>
+      <c r="B9" s="9">
+        <v>10697734</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>77</v>
@@ -3317,13 +3299,13 @@
         <v>79</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G9" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="I9" s="12" t="s">
         <v>83</v>
@@ -3378,13 +3360,13 @@
         <v>91</v>
       </c>
       <c r="Z9" s="12" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="AA9" s="8" t="s">
         <v>139</v>
       </c>
       <c r="AB9" s="8" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="AC9" s="8" t="s">
         <v>95</v>
@@ -3443,7 +3425,7 @@
         <v>104</v>
       </c>
       <c r="AT9" s="18">
-        <v>9561111978</v>
+        <v>9561114596</v>
       </c>
       <c r="AU9" s="13" t="s">
         <v>105</v>
@@ -3458,7 +3440,7 @@
         <v>107</v>
       </c>
       <c r="AY9" s="19">
-        <v>143232874</v>
+        <v>142912906</v>
       </c>
       <c r="AZ9" s="13" t="s">
         <v>105</v>
@@ -3527,10 +3509,10 @@
         <v>79</v>
       </c>
       <c r="BV9" s="20" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="BW9" s="20" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="BX9" s="20">
         <v>211</v>
@@ -3547,10 +3529,10 @@
     </row>
     <row r="10" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C10" s="8" t="s">
         <v>77</v>
@@ -3562,13 +3544,13 @@
         <v>79</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="G10" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="I10" s="12" t="s">
         <v>83</v>
@@ -3629,7 +3611,7 @@
         <v>93</v>
       </c>
       <c r="AB10" s="8" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="AC10" s="8" t="s">
         <v>140</v>
@@ -3671,7 +3653,7 @@
         <v>102</v>
       </c>
       <c r="AO10" s="8" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="AP10" s="11">
         <v>100</v>
@@ -3687,7 +3669,7 @@
         <v>104</v>
       </c>
       <c r="AT10" s="18">
-        <v>9561115146</v>
+        <v>9561116301</v>
       </c>
       <c r="AU10" s="13" t="s">
         <v>105</v>
@@ -3702,7 +3684,7 @@
         <v>107</v>
       </c>
       <c r="AY10" s="19">
-        <v>143222875</v>
+        <v>142902907</v>
       </c>
       <c r="AZ10" s="13" t="s">
         <v>105</v>
@@ -3741,10 +3723,10 @@
         <v>79</v>
       </c>
       <c r="BL10" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="BM10" s="14" t="s">
         <v>153</v>
-      </c>
-      <c r="BM10" s="14" t="s">
-        <v>154</v>
       </c>
       <c r="BN10" s="14" t="s">
         <v>117</v>
@@ -3762,7 +3744,7 @@
         <v>2024</v>
       </c>
       <c r="BS10" s="14" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="BT10" s="14" t="s">
         <v>120</v>
@@ -3771,10 +3753,10 @@
         <v>79</v>
       </c>
       <c r="BV10" s="20" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="BW10" s="20" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="BX10" s="20">
         <v>213</v>
@@ -3791,10 +3773,10 @@
     </row>
     <row r="11" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>205</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>206</v>
+        <v>201</v>
+      </c>
+      <c r="B11" s="9">
+        <v>10697736</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>77</v>
@@ -3806,13 +3788,13 @@
         <v>79</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="G11" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H11" s="12" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="I11" s="12" t="s">
         <v>83</v>
@@ -3867,13 +3849,13 @@
         <v>91</v>
       </c>
       <c r="Z11" s="12" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="AA11" s="8" t="s">
         <v>93</v>
       </c>
       <c r="AB11" s="8" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="AC11" s="8" t="s">
         <v>95</v>
@@ -3931,7 +3913,7 @@
         <v>104</v>
       </c>
       <c r="AT11" s="18">
-        <v>9561118171</v>
+        <v>9561113419</v>
       </c>
       <c r="AU11" s="13" t="s">
         <v>105</v>
@@ -3946,7 +3928,7 @@
         <v>107</v>
       </c>
       <c r="AY11" s="19">
-        <v>143212876</v>
+        <v>142892908</v>
       </c>
       <c r="AZ11" s="13" t="s">
         <v>105</v>
@@ -4015,10 +3997,10 @@
         <v>79</v>
       </c>
       <c r="BV11" s="20" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="BW11" s="20" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="BX11" s="20">
         <v>201</v>
@@ -4035,10 +4017,10 @@
     </row>
     <row r="12" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>213</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>214</v>
+        <v>208</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>209</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>77</v>
@@ -4050,13 +4032,13 @@
         <v>79</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="G12" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H12" s="12" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="I12" s="12" t="s">
         <v>83</v>
@@ -4117,7 +4099,7 @@
         <v>139</v>
       </c>
       <c r="AB12" s="8" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="AC12" s="8" t="s">
         <v>140</v>
@@ -4160,7 +4142,7 @@
         <v>102</v>
       </c>
       <c r="AO12" s="8" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="AP12" s="11">
         <v>100</v>
@@ -4176,7 +4158,7 @@
         <v>104</v>
       </c>
       <c r="AT12" s="18">
-        <v>9561111505</v>
+        <v>9561111879</v>
       </c>
       <c r="AU12" s="13" t="s">
         <v>105</v>
@@ -4191,7 +4173,7 @@
         <v>107</v>
       </c>
       <c r="AY12" s="19">
-        <v>143202877</v>
+        <v>142882909</v>
       </c>
       <c r="AZ12" s="13" t="s">
         <v>105</v>
@@ -4230,10 +4212,10 @@
         <v>79</v>
       </c>
       <c r="BL12" s="14" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="BM12" s="14" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="BN12" s="14" t="s">
         <v>117</v>
@@ -4251,7 +4233,7 @@
         <v>2000</v>
       </c>
       <c r="BS12" s="14" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="BT12" s="14" t="s">
         <v>120</v>
@@ -4260,10 +4242,10 @@
         <v>79</v>
       </c>
       <c r="BV12" s="20" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="BW12" s="20" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="BX12" s="20">
         <v>213</v>
@@ -4280,10 +4262,10 @@
     </row>
     <row r="13" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>221</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>222</v>
+        <v>216</v>
+      </c>
+      <c r="B13" s="9">
+        <v>10697738</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>77</v>
@@ -4295,13 +4277,13 @@
         <v>79</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="G13" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H13" s="12" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="I13" s="12" t="s">
         <v>83</v>
@@ -4356,13 +4338,13 @@
         <v>91</v>
       </c>
       <c r="Z13" s="12" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="AA13" s="8" t="s">
         <v>139</v>
       </c>
       <c r="AB13" s="8" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="AC13" s="8" t="s">
         <v>95</v>
@@ -4421,7 +4403,7 @@
         <v>104</v>
       </c>
       <c r="AT13" s="18">
-        <v>9561112825</v>
+        <v>9561119304</v>
       </c>
       <c r="AU13" s="13" t="s">
         <v>105</v>
@@ -4436,7 +4418,7 @@
         <v>107</v>
       </c>
       <c r="AY13" s="19">
-        <v>143192878</v>
+        <v>142872910</v>
       </c>
       <c r="AZ13" s="13" t="s">
         <v>105</v>
@@ -4505,10 +4487,10 @@
         <v>79</v>
       </c>
       <c r="BV13" s="20" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="BW13" s="20" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="BX13" s="20">
         <v>209</v>
@@ -4525,10 +4507,10 @@
     </row>
     <row r="14" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>77</v>
@@ -4540,13 +4522,13 @@
         <v>79</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="G14" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H14" s="12" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="I14" s="12" t="s">
         <v>83</v>
@@ -4607,7 +4589,7 @@
         <v>93</v>
       </c>
       <c r="AB14" s="8" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="AC14" s="8" t="s">
         <v>140</v>
@@ -4649,7 +4631,7 @@
         <v>102</v>
       </c>
       <c r="AO14" s="8" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="AP14" s="11">
         <v>100</v>
@@ -4665,7 +4647,7 @@
         <v>104</v>
       </c>
       <c r="AT14" s="18">
-        <v>9561111098</v>
+        <v>9561118809</v>
       </c>
       <c r="AU14" s="13" t="s">
         <v>105</v>
@@ -4680,7 +4662,7 @@
         <v>107</v>
       </c>
       <c r="AY14" s="19">
-        <v>143182879</v>
+        <v>142862911</v>
       </c>
       <c r="AZ14" s="13" t="s">
         <v>105</v>
@@ -4749,10 +4731,10 @@
         <v>79</v>
       </c>
       <c r="BV14" s="20" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="BW14" s="20" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="BX14" s="20">
         <v>211</v>
@@ -4769,10 +4751,10 @@
     </row>
     <row r="15" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>77</v>
@@ -4784,13 +4766,13 @@
         <v>79</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="G15" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H15" s="12" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="I15" s="12" t="s">
         <v>83</v>
@@ -4851,7 +4833,7 @@
         <v>139</v>
       </c>
       <c r="AB15" s="8" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="AC15" s="8" t="s">
         <v>95</v>
@@ -4894,7 +4876,7 @@
         <v>102</v>
       </c>
       <c r="AO15" s="8" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="AP15" s="11">
         <v>100</v>
@@ -4910,7 +4892,7 @@
         <v>104</v>
       </c>
       <c r="AT15" s="18">
-        <v>9561115069</v>
+        <v>9561117709</v>
       </c>
       <c r="AU15" s="13" t="s">
         <v>105</v>
@@ -4925,7 +4907,7 @@
         <v>107</v>
       </c>
       <c r="AY15" s="19">
-        <v>143172880</v>
+        <v>142852912</v>
       </c>
       <c r="AZ15" s="13" t="s">
         <v>105</v>
@@ -4964,10 +4946,10 @@
         <v>79</v>
       </c>
       <c r="BL15" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="BM15" s="14" t="s">
         <v>153</v>
-      </c>
-      <c r="BM15" s="14" t="s">
-        <v>154</v>
       </c>
       <c r="BN15" s="14" t="s">
         <v>117</v>
@@ -4985,7 +4967,7 @@
         <v>2024</v>
       </c>
       <c r="BS15" s="14" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="BT15" s="14" t="s">
         <v>120</v>
@@ -4994,10 +4976,10 @@
         <v>79</v>
       </c>
       <c r="BV15" s="20" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="BW15" s="20" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="BX15" s="20">
         <v>213</v>
@@ -5014,10 +4996,10 @@
     </row>
     <row r="16" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="C16" s="8" t="s">
         <v>77</v>
@@ -5029,13 +5011,13 @@
         <v>79</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="G16" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H16" s="12" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="I16" s="12" t="s">
         <v>83</v>
@@ -5138,7 +5120,7 @@
         <v>102</v>
       </c>
       <c r="AO16" s="8" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="AP16" s="11">
         <v>100</v>
@@ -5154,7 +5136,7 @@
         <v>104</v>
       </c>
       <c r="AT16" s="18">
-        <v>9561114101</v>
+        <v>9561118666</v>
       </c>
       <c r="AU16" s="13" t="s">
         <v>105</v>
@@ -5169,7 +5151,7 @@
         <v>107</v>
       </c>
       <c r="AY16" s="19">
-        <v>143162881</v>
+        <v>142842913</v>
       </c>
       <c r="AZ16" s="13" t="s">
         <v>105</v>
@@ -5208,10 +5190,10 @@
         <v>79</v>
       </c>
       <c r="BL16" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="BM16" s="14" t="s">
         <v>153</v>
-      </c>
-      <c r="BM16" s="14" t="s">
-        <v>154</v>
       </c>
       <c r="BN16" s="14" t="s">
         <v>117</v>
@@ -5229,7 +5211,7 @@
         <v>2024</v>
       </c>
       <c r="BS16" s="14" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="BT16" s="14" t="s">
         <v>120</v>
@@ -5238,10 +5220,10 @@
         <v>79</v>
       </c>
       <c r="BV16" s="20" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="BW16" s="20" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="BX16" s="20">
         <v>211</v>

</xml_diff>

<commit_message>
After Spain Completed, dry runs in progress
</commit_message>
<xml_diff>
--- a/Data/Hires/Workday_NewHire_Czechia_Regression_PK14.xlsx
+++ b/Data/Hires/Workday_NewHire_Czechia_Regression_PK14.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{F4FCC049-59D5-4472-9686-D26CD4CF0BF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{3570856E-7080-41D6-B519-93A72A506540}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1068" yWindow="-108" windowWidth="22080" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="997" uniqueCount="244">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -259,7 +259,7 @@
     <t>Test1</t>
   </si>
   <si>
-    <t>10697730</t>
+    <t>10697977</t>
   </si>
   <si>
     <t>Passed</t>
@@ -274,7 +274,7 @@
     <t>CzOne</t>
   </si>
   <si>
-    <t>TwentyFiveAprilSeven</t>
+    <t>TwentyFiveAprilTwentyOne</t>
   </si>
   <si>
     <t>770 272 784</t>
@@ -412,7 +412,7 @@
     <t>Test2</t>
   </si>
   <si>
-    <t>10697766</t>
+    <t>10697978</t>
   </si>
   <si>
     <t>895 Store Management (Jaziz Wezupa (10573442))</t>
@@ -421,7 +421,7 @@
     <t>CzTwo</t>
   </si>
   <si>
-    <t>Auto 25154444</t>
+    <t>Auto 28871520</t>
   </si>
   <si>
     <t>Department Manager_NEW</t>
@@ -442,7 +442,7 @@
     <t>Test3</t>
   </si>
   <si>
-    <t>10697731</t>
+    <t>10697979</t>
   </si>
   <si>
     <t>CzThree</t>
@@ -481,7 +481,7 @@
     <t>CzFour</t>
   </si>
   <si>
-    <t>Auto 9592202</t>
+    <t>Auto 8481544</t>
   </si>
   <si>
     <t>Assistant Store Manager_NEW</t>
@@ -505,7 +505,7 @@
     <t>Test5</t>
   </si>
   <si>
-    <t>Test failed for 'CzFive TwentyFiveAprilSeven' Employee: Errors and AlertsErrorPage Error- You have not entered an amount within the Compensation Guidelines.     (Employee Compensation Event For Hire Employee)AlertPage Alert- "Warning: You have entered an amount that is outside of the range or more than 10% higher than the current salary.  Please re-enter an amount inside the range, below 10% or continue and it will be sent for approval."     (Employee Compensation Event For Hire Employee) &amp; find failed Screenshot Path:-&gt;H:\WorkdayPlaywright/WorkdayFailedScreenshot/2025-04-07T05-12-02-845Z.png</t>
+    <t>Test failed for 'CzFive TwentyFiveAprilTwentyOne' Employee: Errors and AlertsErrorPage Error- You have not entered an amount within the Compensation Guidelines.     (Employee Compensation Event For Hire Employee)AlertPage Alert- "Warning: You have entered an amount that is outside of the range or more than 10% higher than the current salary.  Please re-enter an amount inside the range, below 10% or continue and it will be sent for approval."     (Employee Compensation Event For Hire Employee) &amp; find failed Screenshot Path:-&gt;H:\WorkdayPlaywright/WorkdayFailedScreenshot/2025-04-21T10-56-07-661Z.png</t>
   </si>
   <si>
     <t>Failed</t>
@@ -541,13 +541,19 @@
     <t>Test6</t>
   </si>
   <si>
+    <t>10697996</t>
+  </si>
+  <si>
     <t>CzSix</t>
   </si>
   <si>
+    <t>TwentyFiveAprilTwentyOneA</t>
+  </si>
+  <si>
     <t>771 272 784</t>
   </si>
   <si>
-    <t>Auto 39660385</t>
+    <t>Auto 14139841</t>
   </si>
   <si>
     <t>In-Store Visual Merchandising Manager_NEW</t>
@@ -571,7 +577,7 @@
     <t>Test7</t>
   </si>
   <si>
-    <t>10697733</t>
+    <t>10697981</t>
   </si>
   <si>
     <t>CzSeven</t>
@@ -601,7 +607,7 @@
     <t>773 272 784</t>
   </si>
   <si>
-    <t>Auto 79587467</t>
+    <t>Auto 87502628</t>
   </si>
   <si>
     <t>Store Manager_NEW</t>
@@ -616,7 +622,7 @@
     <t>Test9</t>
   </si>
   <si>
-    <t>10697735</t>
+    <t>10697983</t>
   </si>
   <si>
     <t>CzNine</t>
@@ -643,7 +649,7 @@
     <t>775 272 784</t>
   </si>
   <si>
-    <t>Auto 62280742</t>
+    <t>Auto 57163304</t>
   </si>
   <si>
     <t>Team Manager - Retail_NEW</t>
@@ -658,7 +664,7 @@
     <t>Test11</t>
   </si>
   <si>
-    <t>10697737</t>
+    <t>10697985</t>
   </si>
   <si>
     <t>CzEleven</t>
@@ -688,7 +694,7 @@
     <t>777 272 784</t>
   </si>
   <si>
-    <t>Auto 71162593</t>
+    <t>Auto 72254501</t>
   </si>
   <si>
     <t>In-Store P&amp;C Manager_NEW</t>
@@ -703,7 +709,7 @@
     <t>Test13</t>
   </si>
   <si>
-    <t>10697739</t>
+    <t>10697987</t>
   </si>
   <si>
     <t>CzThirteen</t>
@@ -724,7 +730,7 @@
     <t>Test14</t>
   </si>
   <si>
-    <t>10697741</t>
+    <t>10697988</t>
   </si>
   <si>
     <t>CzFourteen</t>
@@ -742,7 +748,7 @@
     <t>Test15</t>
   </si>
   <si>
-    <t>10697742</t>
+    <t>10697989</t>
   </si>
   <si>
     <t>CzFifteenA</t>
@@ -837,6 +843,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
@@ -844,11 +855,6 @@
       <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
       </patternFill>
     </fill>
   </fills>
@@ -910,7 +916,7 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -926,7 +932,7 @@
     <xf numFmtId="14" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
@@ -949,7 +955,7 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1712,7 +1718,7 @@
         <v>104</v>
       </c>
       <c r="AT2" s="18">
-        <v>9561118391</v>
+        <v>9561114310</v>
       </c>
       <c r="AU2" s="13" t="s">
         <v>105</v>
@@ -1727,7 +1733,7 @@
         <v>107</v>
       </c>
       <c r="AY2" s="19">
-        <v>142982899</v>
+        <v>142472950</v>
       </c>
       <c r="AZ2" s="13" t="s">
         <v>105</v>
@@ -1956,7 +1962,7 @@
         <v>104</v>
       </c>
       <c r="AT3" s="18">
-        <v>9561112374</v>
+        <v>9561112792</v>
       </c>
       <c r="AU3" s="13" t="s">
         <v>105</v>
@@ -1971,7 +1977,7 @@
         <v>107</v>
       </c>
       <c r="AY3" s="19">
-        <v>142972900</v>
+        <v>142462951</v>
       </c>
       <c r="AZ3" s="13" t="s">
         <v>105</v>
@@ -2201,7 +2207,7 @@
         <v>104</v>
       </c>
       <c r="AT4" s="18">
-        <v>9561115564</v>
+        <v>9561119876</v>
       </c>
       <c r="AU4" s="13" t="s">
         <v>105</v>
@@ -2216,7 +2222,7 @@
         <v>107</v>
       </c>
       <c r="AY4" s="19">
-        <v>142962901</v>
+        <v>142452952</v>
       </c>
       <c r="AZ4" s="13" t="s">
         <v>105</v>
@@ -2307,8 +2313,8 @@
       <c r="A5" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="B5" s="9">
-        <v>10697732</v>
+      <c r="B5" s="8">
+        <v>10697980</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>77</v>
@@ -2446,7 +2452,7 @@
         <v>104</v>
       </c>
       <c r="AT5" s="18">
-        <v>9561119909</v>
+        <v>9561115608</v>
       </c>
       <c r="AU5" s="13" t="s">
         <v>105</v>
@@ -2461,7 +2467,7 @@
         <v>107</v>
       </c>
       <c r="AY5" s="19">
-        <v>142952902</v>
+        <v>142442953</v>
       </c>
       <c r="AZ5" s="13" t="s">
         <v>105</v>
@@ -2691,7 +2697,7 @@
         <v>104</v>
       </c>
       <c r="AT6" s="18">
-        <v>9561112110</v>
+        <v>9561112572</v>
       </c>
       <c r="AU6" s="13" t="s">
         <v>105</v>
@@ -2706,7 +2712,7 @@
         <v>107</v>
       </c>
       <c r="AY6" s="19">
-        <v>142942903</v>
+        <v>142432954</v>
       </c>
       <c r="AZ6" s="13" t="s">
         <v>105</v>
@@ -2797,8 +2803,8 @@
       <c r="A7" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="B7" s="9">
-        <v>10697765</v>
+      <c r="B7" s="9" t="s">
+        <v>170</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>77</v>
@@ -2810,13 +2816,13 @@
         <v>79</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>81</v>
+        <v>172</v>
       </c>
       <c r="H7" s="12" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="I7" s="12" t="s">
         <v>83</v>
@@ -2871,13 +2877,13 @@
         <v>91</v>
       </c>
       <c r="Z7" s="12" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="AA7" s="8" t="s">
         <v>93</v>
       </c>
       <c r="AB7" s="8" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="AC7" s="8" t="s">
         <v>140</v>
@@ -2935,7 +2941,7 @@
         <v>104</v>
       </c>
       <c r="AT7" s="18">
-        <v>9561118017</v>
+        <v>9561110372</v>
       </c>
       <c r="AU7" s="13" t="s">
         <v>105</v>
@@ -2950,7 +2956,7 @@
         <v>107</v>
       </c>
       <c r="AY7" s="19">
-        <v>142932904</v>
+        <v>142322965</v>
       </c>
       <c r="AZ7" s="13" t="s">
         <v>105</v>
@@ -2989,10 +2995,10 @@
         <v>79</v>
       </c>
       <c r="BL7" s="14" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="BM7" s="14" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="BN7" s="14" t="s">
         <v>117</v>
@@ -3010,7 +3016,7 @@
         <v>2000</v>
       </c>
       <c r="BS7" s="14" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="BT7" s="14" t="s">
         <v>120</v>
@@ -3019,10 +3025,10 @@
         <v>79</v>
       </c>
       <c r="BV7" s="20" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="BW7" s="20" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="BX7" s="20">
         <v>211</v>
@@ -3039,10 +3045,10 @@
     </row>
     <row r="8" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>77</v>
@@ -3054,13 +3060,13 @@
         <v>79</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="G8" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="I8" s="12" t="s">
         <v>83</v>
@@ -3121,7 +3127,7 @@
         <v>139</v>
       </c>
       <c r="AB8" s="8" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="AC8" s="8" t="s">
         <v>140</v>
@@ -3164,7 +3170,7 @@
         <v>102</v>
       </c>
       <c r="AO8" s="8" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="AP8" s="11">
         <v>100</v>
@@ -3180,7 +3186,7 @@
         <v>104</v>
       </c>
       <c r="AT8" s="18">
-        <v>9561116499</v>
+        <v>9561116279</v>
       </c>
       <c r="AU8" s="13" t="s">
         <v>105</v>
@@ -3195,7 +3201,7 @@
         <v>107</v>
       </c>
       <c r="AY8" s="19">
-        <v>142922905</v>
+        <v>142412956</v>
       </c>
       <c r="AZ8" s="13" t="s">
         <v>105</v>
@@ -3264,10 +3270,10 @@
         <v>79</v>
       </c>
       <c r="BV8" s="20" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="BW8" s="20" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="BX8" s="20">
         <v>213</v>
@@ -3282,12 +3288,12 @@
         <v>125</v>
       </c>
     </row>
-    <row r="9" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B9" s="9">
-        <v>10697734</v>
+        <v>10697997</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>77</v>
@@ -3299,13 +3305,13 @@
         <v>79</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>81</v>
+        <v>172</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="I9" s="12" t="s">
         <v>83</v>
@@ -3360,13 +3366,13 @@
         <v>91</v>
       </c>
       <c r="Z9" s="12" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="AA9" s="8" t="s">
         <v>139</v>
       </c>
       <c r="AB9" s="8" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="AC9" s="8" t="s">
         <v>95</v>
@@ -3425,7 +3431,7 @@
         <v>104</v>
       </c>
       <c r="AT9" s="18">
-        <v>9561114596</v>
+        <v>9561115993</v>
       </c>
       <c r="AU9" s="13" t="s">
         <v>105</v>
@@ -3440,7 +3446,7 @@
         <v>107</v>
       </c>
       <c r="AY9" s="19">
-        <v>142912906</v>
+        <v>142312966</v>
       </c>
       <c r="AZ9" s="13" t="s">
         <v>105</v>
@@ -3509,10 +3515,10 @@
         <v>79</v>
       </c>
       <c r="BV9" s="20" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="BW9" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="BX9" s="20">
         <v>211</v>
@@ -3529,10 +3535,10 @@
     </row>
     <row r="10" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C10" s="8" t="s">
         <v>77</v>
@@ -3544,13 +3550,13 @@
         <v>79</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="G10" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="I10" s="12" t="s">
         <v>83</v>
@@ -3611,7 +3617,7 @@
         <v>93</v>
       </c>
       <c r="AB10" s="8" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="AC10" s="8" t="s">
         <v>140</v>
@@ -3653,7 +3659,7 @@
         <v>102</v>
       </c>
       <c r="AO10" s="8" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="AP10" s="11">
         <v>100</v>
@@ -3669,7 +3675,7 @@
         <v>104</v>
       </c>
       <c r="AT10" s="18">
-        <v>9561116301</v>
+        <v>9561112396</v>
       </c>
       <c r="AU10" s="13" t="s">
         <v>105</v>
@@ -3684,7 +3690,7 @@
         <v>107</v>
       </c>
       <c r="AY10" s="19">
-        <v>142902907</v>
+        <v>142392958</v>
       </c>
       <c r="AZ10" s="13" t="s">
         <v>105</v>
@@ -3753,10 +3759,10 @@
         <v>79</v>
       </c>
       <c r="BV10" s="20" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="BW10" s="20" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="BX10" s="20">
         <v>213</v>
@@ -3773,10 +3779,10 @@
     </row>
     <row r="11" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>201</v>
-      </c>
-      <c r="B11" s="9">
-        <v>10697736</v>
+        <v>203</v>
+      </c>
+      <c r="B11" s="8">
+        <v>10697984</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>77</v>
@@ -3788,13 +3794,13 @@
         <v>79</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="G11" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H11" s="12" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="I11" s="12" t="s">
         <v>83</v>
@@ -3849,13 +3855,13 @@
         <v>91</v>
       </c>
       <c r="Z11" s="12" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="AA11" s="8" t="s">
         <v>93</v>
       </c>
       <c r="AB11" s="8" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="AC11" s="8" t="s">
         <v>95</v>
@@ -3913,7 +3919,7 @@
         <v>104</v>
       </c>
       <c r="AT11" s="18">
-        <v>9561113419</v>
+        <v>9561118193</v>
       </c>
       <c r="AU11" s="13" t="s">
         <v>105</v>
@@ -3928,7 +3934,7 @@
         <v>107</v>
       </c>
       <c r="AY11" s="19">
-        <v>142892908</v>
+        <v>142382959</v>
       </c>
       <c r="AZ11" s="13" t="s">
         <v>105</v>
@@ -3997,10 +4003,10 @@
         <v>79</v>
       </c>
       <c r="BV11" s="20" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="BW11" s="20" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="BX11" s="20">
         <v>201</v>
@@ -4017,10 +4023,10 @@
     </row>
     <row r="12" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>77</v>
@@ -4032,13 +4038,13 @@
         <v>79</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="G12" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H12" s="12" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="I12" s="12" t="s">
         <v>83</v>
@@ -4099,7 +4105,7 @@
         <v>139</v>
       </c>
       <c r="AB12" s="8" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="AC12" s="8" t="s">
         <v>140</v>
@@ -4142,7 +4148,7 @@
         <v>102</v>
       </c>
       <c r="AO12" s="8" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="AP12" s="11">
         <v>100</v>
@@ -4158,7 +4164,7 @@
         <v>104</v>
       </c>
       <c r="AT12" s="18">
-        <v>9561111879</v>
+        <v>9561111802</v>
       </c>
       <c r="AU12" s="13" t="s">
         <v>105</v>
@@ -4173,7 +4179,7 @@
         <v>107</v>
       </c>
       <c r="AY12" s="19">
-        <v>142882909</v>
+        <v>142372960</v>
       </c>
       <c r="AZ12" s="13" t="s">
         <v>105</v>
@@ -4212,10 +4218,10 @@
         <v>79</v>
       </c>
       <c r="BL12" s="14" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="BM12" s="14" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="BN12" s="14" t="s">
         <v>117</v>
@@ -4233,7 +4239,7 @@
         <v>2000</v>
       </c>
       <c r="BS12" s="14" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="BT12" s="14" t="s">
         <v>120</v>
@@ -4242,10 +4248,10 @@
         <v>79</v>
       </c>
       <c r="BV12" s="20" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="BW12" s="20" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="BX12" s="20">
         <v>213</v>
@@ -4262,10 +4268,10 @@
     </row>
     <row r="13" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B13" s="9">
-        <v>10697738</v>
+        <v>10697986</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>77</v>
@@ -4277,13 +4283,13 @@
         <v>79</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="G13" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H13" s="12" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="I13" s="12" t="s">
         <v>83</v>
@@ -4338,13 +4344,13 @@
         <v>91</v>
       </c>
       <c r="Z13" s="12" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="AA13" s="8" t="s">
         <v>139</v>
       </c>
       <c r="AB13" s="8" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="AC13" s="8" t="s">
         <v>95</v>
@@ -4403,7 +4409,7 @@
         <v>104</v>
       </c>
       <c r="AT13" s="18">
-        <v>9561119304</v>
+        <v>9561110174</v>
       </c>
       <c r="AU13" s="13" t="s">
         <v>105</v>
@@ -4418,7 +4424,7 @@
         <v>107</v>
       </c>
       <c r="AY13" s="19">
-        <v>142872910</v>
+        <v>142362961</v>
       </c>
       <c r="AZ13" s="13" t="s">
         <v>105</v>
@@ -4487,10 +4493,10 @@
         <v>79</v>
       </c>
       <c r="BV13" s="20" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="BW13" s="20" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="BX13" s="20">
         <v>209</v>
@@ -4507,10 +4513,10 @@
     </row>
     <row r="14" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>77</v>
@@ -4522,13 +4528,13 @@
         <v>79</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="G14" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H14" s="12" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="I14" s="12" t="s">
         <v>83</v>
@@ -4589,7 +4595,7 @@
         <v>93</v>
       </c>
       <c r="AB14" s="8" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="AC14" s="8" t="s">
         <v>140</v>
@@ -4631,7 +4637,7 @@
         <v>102</v>
       </c>
       <c r="AO14" s="8" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="AP14" s="11">
         <v>100</v>
@@ -4647,7 +4653,7 @@
         <v>104</v>
       </c>
       <c r="AT14" s="18">
-        <v>9561118809</v>
+        <v>9561110350</v>
       </c>
       <c r="AU14" s="13" t="s">
         <v>105</v>
@@ -4662,7 +4668,7 @@
         <v>107</v>
       </c>
       <c r="AY14" s="19">
-        <v>142862911</v>
+        <v>142352962</v>
       </c>
       <c r="AZ14" s="13" t="s">
         <v>105</v>
@@ -4731,10 +4737,10 @@
         <v>79</v>
       </c>
       <c r="BV14" s="20" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="BW14" s="20" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="BX14" s="20">
         <v>211</v>
@@ -4751,10 +4757,10 @@
     </row>
     <row r="15" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>77</v>
@@ -4766,13 +4772,13 @@
         <v>79</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="G15" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H15" s="12" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="I15" s="12" t="s">
         <v>83</v>
@@ -4833,7 +4839,7 @@
         <v>139</v>
       </c>
       <c r="AB15" s="8" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="AC15" s="8" t="s">
         <v>95</v>
@@ -4876,7 +4882,7 @@
         <v>102</v>
       </c>
       <c r="AO15" s="8" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="AP15" s="11">
         <v>100</v>
@@ -4892,7 +4898,7 @@
         <v>104</v>
       </c>
       <c r="AT15" s="18">
-        <v>9561117709</v>
+        <v>9561110284</v>
       </c>
       <c r="AU15" s="13" t="s">
         <v>105</v>
@@ -4907,7 +4913,7 @@
         <v>107</v>
       </c>
       <c r="AY15" s="19">
-        <v>142852912</v>
+        <v>142342963</v>
       </c>
       <c r="AZ15" s="13" t="s">
         <v>105</v>
@@ -4976,10 +4982,10 @@
         <v>79</v>
       </c>
       <c r="BV15" s="20" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="BW15" s="20" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="BX15" s="20">
         <v>213</v>
@@ -4996,10 +5002,10 @@
     </row>
     <row r="16" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C16" s="8" t="s">
         <v>77</v>
@@ -5011,13 +5017,13 @@
         <v>79</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="G16" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H16" s="12" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="I16" s="12" t="s">
         <v>83</v>
@@ -5120,7 +5126,7 @@
         <v>102</v>
       </c>
       <c r="AO16" s="8" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="AP16" s="11">
         <v>100</v>
@@ -5136,7 +5142,7 @@
         <v>104</v>
       </c>
       <c r="AT16" s="18">
-        <v>9561118666</v>
+        <v>9561114486</v>
       </c>
       <c r="AU16" s="13" t="s">
         <v>105</v>
@@ -5151,7 +5157,7 @@
         <v>107</v>
       </c>
       <c r="AY16" s="19">
-        <v>142842913</v>
+        <v>142332964</v>
       </c>
       <c r="AZ16" s="13" t="s">
         <v>105</v>
@@ -5220,10 +5226,10 @@
         <v>79</v>
       </c>
       <c r="BV16" s="20" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="BW16" s="20" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="BX16" s="20">
         <v>211</v>

</xml_diff>

<commit_message>
Portugal Script Maintenance Completed
</commit_message>
<xml_diff>
--- a/Data/Hires/Workday_NewHire_Czechia_Regression_PK14.xlsx
+++ b/Data/Hires/Workday_NewHire_Czechia_Regression_PK14.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{3570856E-7080-41D6-B519-93A72A506540}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69A62D28-FF03-4774-8684-9F6F942647F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1068" yWindow="-108" windowWidth="22080" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11,7 +11,6 @@
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -29,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="997" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="997" uniqueCount="245">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -259,7 +258,7 @@
     <t>Test1</t>
   </si>
   <si>
-    <t>10697977</t>
+    <t>10698112</t>
   </si>
   <si>
     <t>Passed</t>
@@ -274,7 +273,7 @@
     <t>CzOne</t>
   </si>
   <si>
-    <t>TwentyFiveAprilTwentyOne</t>
+    <t>TwentyFiveMayFive</t>
   </si>
   <si>
     <t>770 272 784</t>
@@ -412,16 +411,13 @@
     <t>Test2</t>
   </si>
   <si>
-    <t>10697978</t>
-  </si>
-  <si>
     <t>895 Store Management (Jaziz Wezupa (10573442))</t>
   </si>
   <si>
     <t>CzTwo</t>
   </si>
   <si>
-    <t>Auto 28871520</t>
+    <t>Auto 61082075</t>
   </si>
   <si>
     <t>Department Manager_NEW</t>
@@ -442,7 +438,7 @@
     <t>Test3</t>
   </si>
   <si>
-    <t>10697979</t>
+    <t>10698115</t>
   </si>
   <si>
     <t>CzThree</t>
@@ -481,7 +477,7 @@
     <t>CzFour</t>
   </si>
   <si>
-    <t>Auto 8481544</t>
+    <t>Auto 61248675</t>
   </si>
   <si>
     <t>Assistant Store Manager_NEW</t>
@@ -505,7 +501,7 @@
     <t>Test5</t>
   </si>
   <si>
-    <t>Test failed for 'CzFive TwentyFiveAprilTwentyOne' Employee: Errors and AlertsErrorPage Error- You have not entered an amount within the Compensation Guidelines.     (Employee Compensation Event For Hire Employee)AlertPage Alert- "Warning: You have entered an amount that is outside of the range or more than 10% higher than the current salary.  Please re-enter an amount inside the range, below 10% or continue and it will be sent for approval."     (Employee Compensation Event For Hire Employee) &amp; find failed Screenshot Path:-&gt;H:\WorkdayPlaywright/WorkdayFailedScreenshot/2025-04-21T10-56-07-661Z.png</t>
+    <t>Test failed for 'CzFive TwentyFiveMayFive' Employee: Errors and AlertsErrorPage Error- You have not entered an amount within the Compensation Guidelines.     (Employee Compensation Event For Hire Employee)AlertPage Alert- "Warning: You have entered an amount that is outside of the range or more than 10% higher than the current salary.  Please re-enter an amount inside the range, below 10% or continue and it will be sent for approval."     (Employee Compensation Event For Hire Employee) &amp; find failed Screenshot Path:-&gt;H:\WorkdayPlaywright/WorkdayFailedScreenshot/2025-05-05T04-08-23-543Z.png</t>
   </si>
   <si>
     <t>Failed</t>
@@ -541,19 +537,16 @@
     <t>Test6</t>
   </si>
   <si>
-    <t>10697996</t>
+    <t>Test failed for 'CzSix TwentyFiveMayFive' Employee:{}TypeError: Cannot read properties of undefined (reading 'toString')</t>
   </si>
   <si>
     <t>CzSix</t>
   </si>
   <si>
-    <t>TwentyFiveAprilTwentyOneA</t>
-  </si>
-  <si>
     <t>771 272 784</t>
   </si>
   <si>
-    <t>Auto 14139841</t>
+    <t>Auto 33115070</t>
   </si>
   <si>
     <t>In-Store Visual Merchandising Manager_NEW</t>
@@ -577,12 +570,18 @@
     <t>Test7</t>
   </si>
   <si>
-    <t>10697981</t>
+    <t xml:space="preserve">Test failed for 'CzSeven TwentyFiveMayFiveA' Employee:{Jaziz Wezupa }TimeoutError: locator.click: Timeout 30000ms exceeded.
+Call log:
+  [2m- waiting for getByRole('button', { name: 'Add a Photo', exact: true })[22m
+</t>
   </si>
   <si>
     <t>CzSeven</t>
   </si>
   <si>
+    <t>TwentyFiveMayFiveA</t>
+  </si>
+  <si>
     <t>772 272 784</t>
   </si>
   <si>
@@ -607,7 +606,7 @@
     <t>773 272 784</t>
   </si>
   <si>
-    <t>Auto 87502628</t>
+    <t>Auto 98086062</t>
   </si>
   <si>
     <t>Store Manager_NEW</t>
@@ -622,7 +621,7 @@
     <t>Test9</t>
   </si>
   <si>
-    <t>10697983</t>
+    <t>10698126</t>
   </si>
   <si>
     <t>CzNine</t>
@@ -643,13 +642,16 @@
     <t>Test10</t>
   </si>
   <si>
+    <t>10698120</t>
+  </si>
+  <si>
     <t>CzTen</t>
   </si>
   <si>
     <t>775 272 784</t>
   </si>
   <si>
-    <t>Auto 57163304</t>
+    <t>Auto 98224954</t>
   </si>
   <si>
     <t>Team Manager - Retail_NEW</t>
@@ -664,7 +666,7 @@
     <t>Test11</t>
   </si>
   <si>
-    <t>10697985</t>
+    <t>10698121</t>
   </si>
   <si>
     <t>CzEleven</t>
@@ -694,7 +696,7 @@
     <t>777 272 784</t>
   </si>
   <si>
-    <t>Auto 72254501</t>
+    <t>Auto 27609376</t>
   </si>
   <si>
     <t>In-Store P&amp;C Manager_NEW</t>
@@ -709,7 +711,7 @@
     <t>Test13</t>
   </si>
   <si>
-    <t>10697987</t>
+    <t>10698123</t>
   </si>
   <si>
     <t>CzThirteen</t>
@@ -730,7 +732,7 @@
     <t>Test14</t>
   </si>
   <si>
-    <t>10697988</t>
+    <t>10698124</t>
   </si>
   <si>
     <t>CzFourteen</t>
@@ -748,10 +750,10 @@
     <t>Test15</t>
   </si>
   <si>
-    <t>10697989</t>
-  </si>
-  <si>
-    <t>CzFifteenA</t>
+    <t>10698125</t>
+  </si>
+  <si>
+    <t>CzFifteen</t>
   </si>
   <si>
     <t>255 Stockroom</t>
@@ -761,6 +763,9 @@
   </si>
   <si>
     <t>Onovo</t>
+  </si>
+  <si>
+    <t>TwentyFiveMayFiveB</t>
   </si>
 </sst>
 </file>
@@ -843,11 +848,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
@@ -855,6 +855,11 @@
       <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
       </patternFill>
     </fill>
   </fills>
@@ -916,7 +921,7 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -932,7 +937,7 @@
     <xf numFmtId="14" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
@@ -955,7 +960,7 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1718,7 +1723,7 @@
         <v>104</v>
       </c>
       <c r="AT2" s="18">
-        <v>9561114310</v>
+        <v>9361115379</v>
       </c>
       <c r="AU2" s="13" t="s">
         <v>105</v>
@@ -1733,7 +1738,7 @@
         <v>107</v>
       </c>
       <c r="AY2" s="19">
-        <v>142472950</v>
+        <v>141992998</v>
       </c>
       <c r="AZ2" s="13" t="s">
         <v>105</v>
@@ -1745,7 +1750,7 @@
         <v>108</v>
       </c>
       <c r="BC2" s="13">
-        <v>35014</v>
+        <v>34284</v>
       </c>
       <c r="BD2" s="17" t="s">
         <v>86</v>
@@ -1824,20 +1829,20 @@
       <c r="A3" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="B3" s="9" t="s">
-        <v>127</v>
+      <c r="B3" s="9">
+        <v>10698114</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>77</v>
       </c>
       <c r="D3" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="F3" s="8" t="s">
         <v>128</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>129</v>
       </c>
       <c r="G3" s="12" t="s">
         <v>81</v>
@@ -1898,13 +1903,13 @@
         <v>91</v>
       </c>
       <c r="Z3" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="AA3" s="8" t="s">
         <v>93</v>
       </c>
       <c r="AB3" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AC3" s="8" t="s">
         <v>95</v>
@@ -1943,10 +1948,10 @@
         <v>45597</v>
       </c>
       <c r="AN3" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="AO3" s="8" t="s">
         <v>132</v>
-      </c>
-      <c r="AO3" s="8" t="s">
-        <v>133</v>
       </c>
       <c r="AP3" s="11">
         <v>100</v>
@@ -1962,7 +1967,7 @@
         <v>104</v>
       </c>
       <c r="AT3" s="18">
-        <v>9561112792</v>
+        <v>9361114774</v>
       </c>
       <c r="AU3" s="13" t="s">
         <v>105</v>
@@ -1977,7 +1982,7 @@
         <v>107</v>
       </c>
       <c r="AY3" s="19">
-        <v>142462951</v>
+        <v>141982999</v>
       </c>
       <c r="AZ3" s="13" t="s">
         <v>105</v>
@@ -1989,7 +1994,7 @@
         <v>108</v>
       </c>
       <c r="BC3" s="13">
-        <v>35014</v>
+        <v>34284</v>
       </c>
       <c r="BD3" s="17" t="s">
         <v>86</v>
@@ -2046,10 +2051,10 @@
         <v>79</v>
       </c>
       <c r="BV3" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="BW3" s="20" t="s">
         <v>134</v>
-      </c>
-      <c r="BW3" s="20" t="s">
-        <v>135</v>
       </c>
       <c r="BX3" s="20">
         <v>201</v>
@@ -2066,10 +2071,10 @@
     </row>
     <row r="4" spans="1:92" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="8" t="s">
         <v>136</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>137</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>77</v>
@@ -2081,7 +2086,7 @@
         <v>79</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G4" s="12" t="s">
         <v>81</v>
@@ -2145,13 +2150,13 @@
         <v>92</v>
       </c>
       <c r="AA4" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AB4" s="8" t="s">
         <v>94</v>
       </c>
       <c r="AC4" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AD4" s="11" t="s">
         <v>96</v>
@@ -2160,7 +2165,7 @@
         <v>97</v>
       </c>
       <c r="AF4" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="AG4" s="16">
         <v>20</v>
@@ -2191,7 +2196,7 @@
         <v>102</v>
       </c>
       <c r="AO4" s="8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AP4" s="11">
         <v>100</v>
@@ -2207,7 +2212,7 @@
         <v>104</v>
       </c>
       <c r="AT4" s="18">
-        <v>9561119876</v>
+        <v>9361116116</v>
       </c>
       <c r="AU4" s="13" t="s">
         <v>105</v>
@@ -2222,7 +2227,7 @@
         <v>107</v>
       </c>
       <c r="AY4" s="19">
-        <v>142452952</v>
+        <v>141973000</v>
       </c>
       <c r="AZ4" s="13" t="s">
         <v>105</v>
@@ -2234,7 +2239,7 @@
         <v>108</v>
       </c>
       <c r="BC4" s="13">
-        <v>35014</v>
+        <v>34284</v>
       </c>
       <c r="BD4" s="17" t="s">
         <v>86</v>
@@ -2261,10 +2266,10 @@
         <v>79</v>
       </c>
       <c r="BL4" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="BM4" s="14" t="s">
         <v>143</v>
-      </c>
-      <c r="BM4" s="14" t="s">
-        <v>144</v>
       </c>
       <c r="BN4" s="14" t="s">
         <v>117</v>
@@ -2282,7 +2287,7 @@
         <v>1991</v>
       </c>
       <c r="BS4" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="BT4" s="14" t="s">
         <v>120</v>
@@ -2291,10 +2296,10 @@
         <v>79</v>
       </c>
       <c r="BV4" s="20" t="s">
+        <v>145</v>
+      </c>
+      <c r="BW4" s="20" t="s">
         <v>146</v>
-      </c>
-      <c r="BW4" s="20" t="s">
-        <v>147</v>
       </c>
       <c r="BX4" s="20">
         <v>213</v>
@@ -2311,22 +2316,22 @@
     </row>
     <row r="5" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="B5" s="8">
-        <v>10697980</v>
+        <v>147</v>
+      </c>
+      <c r="B5" s="9">
+        <v>10698116</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>77</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E5" s="11" t="s">
         <v>79</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G5" s="12" t="s">
         <v>81</v>
@@ -2387,13 +2392,13 @@
         <v>91</v>
       </c>
       <c r="Z5" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="AA5" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="AB5" s="8" t="s">
         <v>150</v>
-      </c>
-      <c r="AA5" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="AB5" s="8" t="s">
-        <v>151</v>
       </c>
       <c r="AC5" s="8" t="s">
         <v>95</v>
@@ -2433,10 +2438,10 @@
         <v>45597</v>
       </c>
       <c r="AN5" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="AO5" s="8" t="s">
         <v>132</v>
-      </c>
-      <c r="AO5" s="8" t="s">
-        <v>133</v>
       </c>
       <c r="AP5" s="11">
         <v>100</v>
@@ -2452,7 +2457,7 @@
         <v>104</v>
       </c>
       <c r="AT5" s="18">
-        <v>9561115608</v>
+        <v>9361111947</v>
       </c>
       <c r="AU5" s="13" t="s">
         <v>105</v>
@@ -2467,7 +2472,7 @@
         <v>107</v>
       </c>
       <c r="AY5" s="19">
-        <v>142442953</v>
+        <v>141963001</v>
       </c>
       <c r="AZ5" s="13" t="s">
         <v>105</v>
@@ -2479,7 +2484,7 @@
         <v>108</v>
       </c>
       <c r="BC5" s="13">
-        <v>35014</v>
+        <v>34284</v>
       </c>
       <c r="BD5" s="17" t="s">
         <v>86</v>
@@ -2506,10 +2511,10 @@
         <v>79</v>
       </c>
       <c r="BL5" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="BM5" s="14" t="s">
         <v>152</v>
-      </c>
-      <c r="BM5" s="14" t="s">
-        <v>153</v>
       </c>
       <c r="BN5" s="14" t="s">
         <v>117</v>
@@ -2527,7 +2532,7 @@
         <v>2024</v>
       </c>
       <c r="BS5" s="14" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="BT5" s="14" t="s">
         <v>120</v>
@@ -2536,10 +2541,10 @@
         <v>79</v>
       </c>
       <c r="BV5" s="20" t="s">
+        <v>154</v>
+      </c>
+      <c r="BW5" s="20" t="s">
         <v>155</v>
-      </c>
-      <c r="BW5" s="20" t="s">
-        <v>156</v>
       </c>
       <c r="BX5" s="20">
         <v>207</v>
@@ -2556,13 +2561,13 @@
     </row>
     <row r="6" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="B6" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="C6" s="8" t="s">
         <v>158</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>159</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>78</v>
@@ -2571,7 +2576,7 @@
         <v>79</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G6" s="12" t="s">
         <v>81</v>
@@ -2635,22 +2640,22 @@
         <v>92</v>
       </c>
       <c r="AA6" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="AB6" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="AB6" s="8" t="s">
-        <v>162</v>
-      </c>
       <c r="AC6" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AD6" s="11" t="s">
         <v>96</v>
       </c>
       <c r="AE6" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="AF6" s="8" t="s">
         <v>163</v>
-      </c>
-      <c r="AF6" s="8" t="s">
-        <v>164</v>
       </c>
       <c r="AG6" s="16">
         <v>16</v>
@@ -2660,7 +2665,7 @@
         <v>45962</v>
       </c>
       <c r="AI6" s="12" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AJ6" s="12" t="s">
         <v>101</v>
@@ -2681,7 +2686,7 @@
         <v>102</v>
       </c>
       <c r="AO6" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="AP6" s="11">
         <v>100</v>
@@ -2697,7 +2702,7 @@
         <v>104</v>
       </c>
       <c r="AT6" s="18">
-        <v>9561112572</v>
+        <v>9361114928</v>
       </c>
       <c r="AU6" s="13" t="s">
         <v>105</v>
@@ -2712,7 +2717,7 @@
         <v>107</v>
       </c>
       <c r="AY6" s="19">
-        <v>142432954</v>
+        <v>141953002</v>
       </c>
       <c r="AZ6" s="13" t="s">
         <v>105</v>
@@ -2724,7 +2729,7 @@
         <v>108</v>
       </c>
       <c r="BC6" s="13">
-        <v>35014</v>
+        <v>34284</v>
       </c>
       <c r="BD6" s="17" t="s">
         <v>86</v>
@@ -2781,10 +2786,10 @@
         <v>79</v>
       </c>
       <c r="BV6" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="BW6" s="20" t="s">
         <v>167</v>
-      </c>
-      <c r="BW6" s="20" t="s">
-        <v>168</v>
       </c>
       <c r="BX6" s="20">
         <v>211</v>
@@ -2799,30 +2804,30 @@
         <v>125</v>
       </c>
     </row>
-    <row r="7" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="C7" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="F7" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="C7" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>128</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="F7" s="8" t="s">
+      <c r="G7" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="H7" s="12" t="s">
         <v>171</v>
-      </c>
-      <c r="G7" s="12" t="s">
-        <v>172</v>
-      </c>
-      <c r="H7" s="12" t="s">
-        <v>173</v>
       </c>
       <c r="I7" s="12" t="s">
         <v>83</v>
@@ -2877,16 +2882,16 @@
         <v>91</v>
       </c>
       <c r="Z7" s="12" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="AA7" s="8" t="s">
         <v>93</v>
       </c>
       <c r="AB7" s="8" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="AC7" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AD7" s="11" t="s">
         <v>96</v>
@@ -2922,10 +2927,10 @@
         <v>45597</v>
       </c>
       <c r="AN7" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="AO7" s="8" t="s">
         <v>132</v>
-      </c>
-      <c r="AO7" s="8" t="s">
-        <v>133</v>
       </c>
       <c r="AP7" s="11">
         <v>100</v>
@@ -2941,7 +2946,7 @@
         <v>104</v>
       </c>
       <c r="AT7" s="18">
-        <v>9561110372</v>
+        <v>9361115577</v>
       </c>
       <c r="AU7" s="13" t="s">
         <v>105</v>
@@ -2956,7 +2961,7 @@
         <v>107</v>
       </c>
       <c r="AY7" s="19">
-        <v>142322965</v>
+        <v>141943003</v>
       </c>
       <c r="AZ7" s="13" t="s">
         <v>105</v>
@@ -2968,7 +2973,7 @@
         <v>108</v>
       </c>
       <c r="BC7" s="13">
-        <v>35014</v>
+        <v>34284</v>
       </c>
       <c r="BD7" s="17" t="s">
         <v>86</v>
@@ -2995,10 +3000,10 @@
         <v>79</v>
       </c>
       <c r="BL7" s="14" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="BM7" s="14" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="BN7" s="14" t="s">
         <v>117</v>
@@ -3016,7 +3021,7 @@
         <v>2000</v>
       </c>
       <c r="BS7" s="14" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="BT7" s="14" t="s">
         <v>120</v>
@@ -3025,10 +3030,10 @@
         <v>79</v>
       </c>
       <c r="BV7" s="20" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="BW7" s="20" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="BX7" s="20">
         <v>211</v>
@@ -3043,15 +3048,15 @@
         <v>125</v>
       </c>
     </row>
-    <row r="8" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>77</v>
+        <v>158</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>78</v>
@@ -3060,13 +3065,13 @@
         <v>79</v>
       </c>
       <c r="F8" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="H8" s="12" t="s">
         <v>183</v>
-      </c>
-      <c r="G8" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="H8" s="12" t="s">
-        <v>184</v>
       </c>
       <c r="I8" s="12" t="s">
         <v>83</v>
@@ -3124,13 +3129,13 @@
         <v>92</v>
       </c>
       <c r="AA8" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="AB8" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="AC8" s="8" t="s">
         <v>139</v>
-      </c>
-      <c r="AB8" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="AC8" s="8" t="s">
-        <v>140</v>
       </c>
       <c r="AD8" s="11" t="s">
         <v>96</v>
@@ -3170,7 +3175,7 @@
         <v>102</v>
       </c>
       <c r="AO8" s="8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AP8" s="11">
         <v>100</v>
@@ -3186,7 +3191,7 @@
         <v>104</v>
       </c>
       <c r="AT8" s="18">
-        <v>9561116279</v>
+        <v>9361114752</v>
       </c>
       <c r="AU8" s="13" t="s">
         <v>105</v>
@@ -3201,7 +3206,7 @@
         <v>107</v>
       </c>
       <c r="AY8" s="19">
-        <v>142412956</v>
+        <v>141933004</v>
       </c>
       <c r="AZ8" s="13" t="s">
         <v>105</v>
@@ -3213,7 +3218,7 @@
         <v>108</v>
       </c>
       <c r="BC8" s="13">
-        <v>35014</v>
+        <v>34284</v>
       </c>
       <c r="BD8" s="17" t="s">
         <v>86</v>
@@ -3270,10 +3275,10 @@
         <v>79</v>
       </c>
       <c r="BV8" s="20" t="s">
+        <v>186</v>
+      </c>
+      <c r="BW8" s="20" t="s">
         <v>187</v>
-      </c>
-      <c r="BW8" s="20" t="s">
-        <v>188</v>
       </c>
       <c r="BX8" s="20">
         <v>213</v>
@@ -3288,30 +3293,30 @@
         <v>125</v>
       </c>
     </row>
-    <row r="9" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B9" s="9">
-        <v>10697997</v>
+        <v>10698117</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>77</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E9" s="11" t="s">
         <v>79</v>
       </c>
       <c r="F9" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="H9" s="12" t="s">
         <v>190</v>
-      </c>
-      <c r="G9" s="12" t="s">
-        <v>172</v>
-      </c>
-      <c r="H9" s="12" t="s">
-        <v>191</v>
       </c>
       <c r="I9" s="12" t="s">
         <v>83</v>
@@ -3366,13 +3371,13 @@
         <v>91</v>
       </c>
       <c r="Z9" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="AA9" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="AB9" s="8" t="s">
         <v>192</v>
-      </c>
-      <c r="AA9" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="AB9" s="8" t="s">
-        <v>193</v>
       </c>
       <c r="AC9" s="8" t="s">
         <v>95</v>
@@ -3412,10 +3417,10 @@
         <v>45597</v>
       </c>
       <c r="AN9" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="AO9" s="8" t="s">
         <v>132</v>
-      </c>
-      <c r="AO9" s="8" t="s">
-        <v>133</v>
       </c>
       <c r="AP9" s="11">
         <v>100</v>
@@ -3431,7 +3436,7 @@
         <v>104</v>
       </c>
       <c r="AT9" s="18">
-        <v>9561115993</v>
+        <v>9361112541</v>
       </c>
       <c r="AU9" s="13" t="s">
         <v>105</v>
@@ -3446,7 +3451,7 @@
         <v>107</v>
       </c>
       <c r="AY9" s="19">
-        <v>142312966</v>
+        <v>141923005</v>
       </c>
       <c r="AZ9" s="13" t="s">
         <v>105</v>
@@ -3458,7 +3463,7 @@
         <v>108</v>
       </c>
       <c r="BC9" s="13">
-        <v>35014</v>
+        <v>34284</v>
       </c>
       <c r="BD9" s="17" t="s">
         <v>86</v>
@@ -3485,10 +3490,10 @@
         <v>79</v>
       </c>
       <c r="BL9" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="BM9" s="14" t="s">
         <v>143</v>
-      </c>
-      <c r="BM9" s="14" t="s">
-        <v>144</v>
       </c>
       <c r="BN9" s="14" t="s">
         <v>117</v>
@@ -3506,7 +3511,7 @@
         <v>1991</v>
       </c>
       <c r="BS9" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="BT9" s="14" t="s">
         <v>120</v>
@@ -3515,10 +3520,10 @@
         <v>79</v>
       </c>
       <c r="BV9" s="20" t="s">
+        <v>193</v>
+      </c>
+      <c r="BW9" s="20" t="s">
         <v>194</v>
-      </c>
-      <c r="BW9" s="20" t="s">
-        <v>195</v>
       </c>
       <c r="BX9" s="20">
         <v>211</v>
@@ -3535,10 +3540,10 @@
     </row>
     <row r="10" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>196</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>197</v>
       </c>
       <c r="C10" s="8" t="s">
         <v>77</v>
@@ -3550,13 +3555,13 @@
         <v>79</v>
       </c>
       <c r="F10" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>182</v>
+      </c>
+      <c r="H10" s="12" t="s">
         <v>198</v>
-      </c>
-      <c r="G10" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="H10" s="12" t="s">
-        <v>199</v>
       </c>
       <c r="I10" s="12" t="s">
         <v>83</v>
@@ -3617,10 +3622,10 @@
         <v>93</v>
       </c>
       <c r="AB10" s="8" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="AC10" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AD10" s="11" t="s">
         <v>96</v>
@@ -3629,7 +3634,7 @@
         <v>97</v>
       </c>
       <c r="AF10" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="AG10" s="16">
         <v>20</v>
@@ -3659,7 +3664,7 @@
         <v>102</v>
       </c>
       <c r="AO10" s="8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AP10" s="11">
         <v>100</v>
@@ -3675,7 +3680,7 @@
         <v>104</v>
       </c>
       <c r="AT10" s="18">
-        <v>9561112396</v>
+        <v>9361113399</v>
       </c>
       <c r="AU10" s="13" t="s">
         <v>105</v>
@@ -3690,7 +3695,7 @@
         <v>107</v>
       </c>
       <c r="AY10" s="19">
-        <v>142392958</v>
+        <v>141913006</v>
       </c>
       <c r="AZ10" s="13" t="s">
         <v>105</v>
@@ -3702,7 +3707,7 @@
         <v>108</v>
       </c>
       <c r="BC10" s="13">
-        <v>35014</v>
+        <v>34284</v>
       </c>
       <c r="BD10" s="17" t="s">
         <v>86</v>
@@ -3729,10 +3734,10 @@
         <v>79</v>
       </c>
       <c r="BL10" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="BM10" s="14" t="s">
         <v>152</v>
-      </c>
-      <c r="BM10" s="14" t="s">
-        <v>153</v>
       </c>
       <c r="BN10" s="14" t="s">
         <v>117</v>
@@ -3750,7 +3755,7 @@
         <v>2024</v>
       </c>
       <c r="BS10" s="14" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="BT10" s="14" t="s">
         <v>120</v>
@@ -3759,10 +3764,10 @@
         <v>79</v>
       </c>
       <c r="BV10" s="20" t="s">
+        <v>200</v>
+      </c>
+      <c r="BW10" s="20" t="s">
         <v>201</v>
-      </c>
-      <c r="BW10" s="20" t="s">
-        <v>202</v>
       </c>
       <c r="BX10" s="20">
         <v>213</v>
@@ -3779,16 +3784,16 @@
     </row>
     <row r="11" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>203</v>
-      </c>
-      <c r="B11" s="8">
-        <v>10697984</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>77</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E11" s="11" t="s">
         <v>79</v>
@@ -3900,10 +3905,10 @@
         <v>45597</v>
       </c>
       <c r="AN11" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="AO11" s="8" t="s">
         <v>132</v>
-      </c>
-      <c r="AO11" s="8" t="s">
-        <v>133</v>
       </c>
       <c r="AP11" s="11">
         <v>100</v>
@@ -3919,7 +3924,7 @@
         <v>104</v>
       </c>
       <c r="AT11" s="18">
-        <v>9561118193</v>
+        <v>9361113927</v>
       </c>
       <c r="AU11" s="13" t="s">
         <v>105</v>
@@ -3934,7 +3939,7 @@
         <v>107</v>
       </c>
       <c r="AY11" s="19">
-        <v>142382959</v>
+        <v>141903007</v>
       </c>
       <c r="AZ11" s="13" t="s">
         <v>105</v>
@@ -3946,7 +3951,7 @@
         <v>108</v>
       </c>
       <c r="BC11" s="13">
-        <v>35014</v>
+        <v>34284</v>
       </c>
       <c r="BD11" s="17" t="s">
         <v>86</v>
@@ -4102,13 +4107,13 @@
         <v>92</v>
       </c>
       <c r="AA12" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AB12" s="8" t="s">
         <v>214</v>
       </c>
       <c r="AC12" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AD12" s="11" t="s">
         <v>96</v>
@@ -4164,7 +4169,7 @@
         <v>104</v>
       </c>
       <c r="AT12" s="18">
-        <v>9561111802</v>
+        <v>9361111078</v>
       </c>
       <c r="AU12" s="13" t="s">
         <v>105</v>
@@ -4179,7 +4184,7 @@
         <v>107</v>
       </c>
       <c r="AY12" s="19">
-        <v>142372960</v>
+        <v>141893008</v>
       </c>
       <c r="AZ12" s="13" t="s">
         <v>105</v>
@@ -4191,7 +4196,7 @@
         <v>108</v>
       </c>
       <c r="BC12" s="13">
-        <v>35014</v>
+        <v>34284</v>
       </c>
       <c r="BD12" s="17" t="s">
         <v>86</v>
@@ -4218,10 +4223,10 @@
         <v>79</v>
       </c>
       <c r="BL12" s="14" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="BM12" s="14" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="BN12" s="14" t="s">
         <v>117</v>
@@ -4239,7 +4244,7 @@
         <v>2000</v>
       </c>
       <c r="BS12" s="14" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="BT12" s="14" t="s">
         <v>120</v>
@@ -4271,13 +4276,13 @@
         <v>218</v>
       </c>
       <c r="B13" s="9">
-        <v>10697986</v>
+        <v>10698122</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>77</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E13" s="11" t="s">
         <v>79</v>
@@ -4347,7 +4352,7 @@
         <v>221</v>
       </c>
       <c r="AA13" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AB13" s="8" t="s">
         <v>222</v>
@@ -4390,10 +4395,10 @@
         <v>45597</v>
       </c>
       <c r="AN13" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="AO13" s="8" t="s">
         <v>132</v>
-      </c>
-      <c r="AO13" s="8" t="s">
-        <v>133</v>
       </c>
       <c r="AP13" s="11">
         <v>100</v>
@@ -4409,7 +4414,7 @@
         <v>104</v>
       </c>
       <c r="AT13" s="18">
-        <v>9561110174</v>
+        <v>9361113476</v>
       </c>
       <c r="AU13" s="13" t="s">
         <v>105</v>
@@ -4424,7 +4429,7 @@
         <v>107</v>
       </c>
       <c r="AY13" s="19">
-        <v>142362961</v>
+        <v>141883009</v>
       </c>
       <c r="AZ13" s="13" t="s">
         <v>105</v>
@@ -4436,7 +4441,7 @@
         <v>108</v>
       </c>
       <c r="BC13" s="13">
-        <v>35014</v>
+        <v>34284</v>
       </c>
       <c r="BD13" s="17" t="s">
         <v>86</v>
@@ -4515,7 +4520,7 @@
       <c r="A14" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="9" t="s">
         <v>226</v>
       </c>
       <c r="C14" s="8" t="s">
@@ -4595,10 +4600,10 @@
         <v>93</v>
       </c>
       <c r="AB14" s="8" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="AC14" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AD14" s="11" t="s">
         <v>96</v>
@@ -4607,7 +4612,7 @@
         <v>97</v>
       </c>
       <c r="AF14" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="AG14" s="16">
         <v>24</v>
@@ -4653,7 +4658,7 @@
         <v>104</v>
       </c>
       <c r="AT14" s="18">
-        <v>9561110350</v>
+        <v>9361115423</v>
       </c>
       <c r="AU14" s="13" t="s">
         <v>105</v>
@@ -4668,7 +4673,7 @@
         <v>107</v>
       </c>
       <c r="AY14" s="19">
-        <v>142352962</v>
+        <v>141873010</v>
       </c>
       <c r="AZ14" s="13" t="s">
         <v>105</v>
@@ -4680,7 +4685,7 @@
         <v>108</v>
       </c>
       <c r="BC14" s="13">
-        <v>35014</v>
+        <v>34284</v>
       </c>
       <c r="BD14" s="17" t="s">
         <v>86</v>
@@ -4707,10 +4712,10 @@
         <v>79</v>
       </c>
       <c r="BL14" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="BM14" s="14" t="s">
         <v>143</v>
-      </c>
-      <c r="BM14" s="14" t="s">
-        <v>144</v>
       </c>
       <c r="BN14" s="14" t="s">
         <v>117</v>
@@ -4728,7 +4733,7 @@
         <v>1991</v>
       </c>
       <c r="BS14" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="BT14" s="14" t="s">
         <v>120</v>
@@ -4759,7 +4764,7 @@
       <c r="A15" s="8" t="s">
         <v>232</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="21" t="s">
         <v>233</v>
       </c>
       <c r="C15" s="8" t="s">
@@ -4836,10 +4841,10 @@
         <v>92</v>
       </c>
       <c r="AA15" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AB15" s="8" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="AC15" s="8" t="s">
         <v>95</v>
@@ -4882,7 +4887,7 @@
         <v>102</v>
       </c>
       <c r="AO15" s="8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AP15" s="11">
         <v>100</v>
@@ -4898,7 +4903,7 @@
         <v>104</v>
       </c>
       <c r="AT15" s="18">
-        <v>9561110284</v>
+        <v>9361112728</v>
       </c>
       <c r="AU15" s="13" t="s">
         <v>105</v>
@@ -4913,7 +4918,7 @@
         <v>107</v>
       </c>
       <c r="AY15" s="19">
-        <v>142342963</v>
+        <v>141863011</v>
       </c>
       <c r="AZ15" s="13" t="s">
         <v>105</v>
@@ -4925,7 +4930,7 @@
         <v>108</v>
       </c>
       <c r="BC15" s="13">
-        <v>35014</v>
+        <v>34284</v>
       </c>
       <c r="BD15" s="17" t="s">
         <v>86</v>
@@ -4952,10 +4957,10 @@
         <v>79</v>
       </c>
       <c r="BL15" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="BM15" s="14" t="s">
         <v>152</v>
-      </c>
-      <c r="BM15" s="14" t="s">
-        <v>153</v>
       </c>
       <c r="BN15" s="14" t="s">
         <v>117</v>
@@ -4973,7 +4978,7 @@
         <v>2024</v>
       </c>
       <c r="BS15" s="14" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="BT15" s="14" t="s">
         <v>120</v>
@@ -5087,7 +5092,7 @@
         <v>94</v>
       </c>
       <c r="AC16" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AD16" s="11" t="s">
         <v>96</v>
@@ -5142,7 +5147,7 @@
         <v>104</v>
       </c>
       <c r="AT16" s="18">
-        <v>9561114486</v>
+        <v>9361115896</v>
       </c>
       <c r="AU16" s="13" t="s">
         <v>105</v>
@@ -5157,7 +5162,7 @@
         <v>107</v>
       </c>
       <c r="AY16" s="19">
-        <v>142332964</v>
+        <v>141853012</v>
       </c>
       <c r="AZ16" s="13" t="s">
         <v>105</v>
@@ -5169,7 +5174,7 @@
         <v>108</v>
       </c>
       <c r="BC16" s="13">
-        <v>35014</v>
+        <v>34284</v>
       </c>
       <c r="BD16" s="17" t="s">
         <v>86</v>
@@ -5196,10 +5201,10 @@
         <v>79</v>
       </c>
       <c r="BL16" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="BM16" s="14" t="s">
         <v>152</v>
-      </c>
-      <c r="BM16" s="14" t="s">
-        <v>153</v>
       </c>
       <c r="BN16" s="14" t="s">
         <v>117</v>
@@ -5217,7 +5222,7 @@
         <v>2024</v>
       </c>
       <c r="BS16" s="14" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="BT16" s="14" t="s">
         <v>120</v>

</xml_diff>

<commit_message>
Belgium Rehire In Progress 9th June'25
</commit_message>
<xml_diff>
--- a/Data/Hires/Workday_NewHire_Czechia_Regression_PK14.xlsx
+++ b/Data/Hires/Workday_NewHire_Czechia_Regression_PK14.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69A62D28-FF03-4774-8684-9F6F942647F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{AADDD124-BE72-4955-B343-E8BD563FC6E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1068" yWindow="-108" windowWidth="22080" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11,6 +11,7 @@
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="997" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="247">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -258,7 +259,7 @@
     <t>Test1</t>
   </si>
   <si>
-    <t>10698112</t>
+    <t>10698205</t>
   </si>
   <si>
     <t>Passed</t>
@@ -273,7 +274,7 @@
     <t>CzOne</t>
   </si>
   <si>
-    <t>TwentyFiveMayFive</t>
+    <t>TwentyFiveMayThirteen</t>
   </si>
   <si>
     <t>770 272 784</t>
@@ -411,13 +412,16 @@
     <t>Test2</t>
   </si>
   <si>
+    <t>10698206</t>
+  </si>
+  <si>
     <t>895 Store Management (Jaziz Wezupa (10573442))</t>
   </si>
   <si>
     <t>CzTwo</t>
   </si>
   <si>
-    <t>Auto 61082075</t>
+    <t>Auto 61241649</t>
   </si>
   <si>
     <t>Department Manager_NEW</t>
@@ -438,7 +442,7 @@
     <t>Test3</t>
   </si>
   <si>
-    <t>10698115</t>
+    <t>10698207</t>
   </si>
   <si>
     <t>CzThree</t>
@@ -474,10 +478,13 @@
     <t>Test4</t>
   </si>
   <si>
+    <t>10698208</t>
+  </si>
+  <si>
     <t>CzFour</t>
   </si>
   <si>
-    <t>Auto 61248675</t>
+    <t>Auto 74699468</t>
   </si>
   <si>
     <t>Assistant Store Manager_NEW</t>
@@ -501,7 +508,7 @@
     <t>Test5</t>
   </si>
   <si>
-    <t>Test failed for 'CzFive TwentyFiveMayFive' Employee: Errors and AlertsErrorPage Error- You have not entered an amount within the Compensation Guidelines.     (Employee Compensation Event For Hire Employee)AlertPage Alert- "Warning: You have entered an amount that is outside of the range or more than 10% higher than the current salary.  Please re-enter an amount inside the range, below 10% or continue and it will be sent for approval."     (Employee Compensation Event For Hire Employee) &amp; find failed Screenshot Path:-&gt;H:\WorkdayPlaywright/WorkdayFailedScreenshot/2025-05-05T04-08-23-543Z.png</t>
+    <t>Test failed for 'CzFive TwentyFiveMayThirteen' Employee: Errors and AlertsErrorPage Error- You have not entered an amount within the Compensation Guidelines.     (Employee Compensation Event For Hire Employee)AlertPage Alert- "Warning: You have entered an amount that is outside of the range or more than 10% higher than the current salary.  Please re-enter an amount inside the range, below 10% or continue and it will be sent for approval."     (Employee Compensation Event For Hire Employee) &amp; find failed Screenshot Path:-&gt;H:\WorkdayPlaywright/WorkdayFailedScreenshot/2025-05-13T04-02-12-107Z.png</t>
   </si>
   <si>
     <t>Failed</t>
@@ -537,7 +544,7 @@
     <t>Test6</t>
   </si>
   <si>
-    <t>Test failed for 'CzSix TwentyFiveMayFive' Employee:{}TypeError: Cannot read properties of undefined (reading 'toString')</t>
+    <t>Test failed for 'CzSix TwentyFiveMayThirteen' Employee:{}TypeError: Cannot read properties of undefined (reading 'toString')</t>
   </si>
   <si>
     <t>CzSix</t>
@@ -546,7 +553,7 @@
     <t>771 272 784</t>
   </si>
   <si>
-    <t>Auto 33115070</t>
+    <t>Auto 28909772</t>
   </si>
   <si>
     <t>In-Store Visual Merchandising Manager_NEW</t>
@@ -570,7 +577,7 @@
     <t>Test7</t>
   </si>
   <si>
-    <t xml:space="preserve">Test failed for 'CzSeven TwentyFiveMayFiveA' Employee:{Jaziz Wezupa }TimeoutError: locator.click: Timeout 30000ms exceeded.
+    <t xml:space="preserve">Test failed for 'CzSeven TwentyFiveMayThirteen' Employee:{Jaziz Wezupa }TimeoutError: locator.click: Timeout 30000ms exceeded.
 Call log:
   [2m- waiting for getByRole('button', { name: 'Add a Photo', exact: true })[22m
 </t>
@@ -579,9 +586,6 @@
     <t>CzSeven</t>
   </si>
   <si>
-    <t>TwentyFiveMayFiveA</t>
-  </si>
-  <si>
     <t>772 272 784</t>
   </si>
   <si>
@@ -600,13 +604,16 @@
     <t>Test8</t>
   </si>
   <si>
+    <t>10698209</t>
+  </si>
+  <si>
     <t>CzEight</t>
   </si>
   <si>
     <t>773 272 784</t>
   </si>
   <si>
-    <t>Auto 98086062</t>
+    <t>Auto 49138040</t>
   </si>
   <si>
     <t>Store Manager_NEW</t>
@@ -621,7 +628,7 @@
     <t>Test9</t>
   </si>
   <si>
-    <t>10698126</t>
+    <t>10698210</t>
   </si>
   <si>
     <t>CzNine</t>
@@ -642,7 +649,7 @@
     <t>Test10</t>
   </si>
   <si>
-    <t>10698120</t>
+    <t>10698211</t>
   </si>
   <si>
     <t>CzTen</t>
@@ -651,7 +658,7 @@
     <t>775 272 784</t>
   </si>
   <si>
-    <t>Auto 98224954</t>
+    <t>Auto 32360845</t>
   </si>
   <si>
     <t>Team Manager - Retail_NEW</t>
@@ -666,7 +673,7 @@
     <t>Test11</t>
   </si>
   <si>
-    <t>10698121</t>
+    <t>10698212</t>
   </si>
   <si>
     <t>CzEleven</t>
@@ -690,13 +697,16 @@
     <t>Test12</t>
   </si>
   <si>
+    <t>Test failed for 'CzTweve TwentyFiveMayThirteen' Employee: Errors and AlertsAlertNational IDs (Row 2)This national identifier you entered is already in use. Verify that the information is accurate. &amp; find failed Screenshot Path:-&gt;H:\WorkdayPlaywright/WorkdayFailedScreenshot/2025-05-13T05-05-28-017Z.png</t>
+  </si>
+  <si>
     <t>CzTweve</t>
   </si>
   <si>
     <t>777 272 784</t>
   </si>
   <si>
-    <t>Auto 27609376</t>
+    <t>Auto 52738901</t>
   </si>
   <si>
     <t>In-Store P&amp;C Manager_NEW</t>
@@ -711,7 +721,7 @@
     <t>Test13</t>
   </si>
   <si>
-    <t>10698123</t>
+    <t>10698214</t>
   </si>
   <si>
     <t>CzThirteen</t>
@@ -732,7 +742,7 @@
     <t>Test14</t>
   </si>
   <si>
-    <t>10698124</t>
+    <t>10698215</t>
   </si>
   <si>
     <t>CzFourteen</t>
@@ -750,7 +760,7 @@
     <t>Test15</t>
   </si>
   <si>
-    <t>10698125</t>
+    <t>10698216</t>
   </si>
   <si>
     <t>CzFifteen</t>
@@ -763,9 +773,6 @@
   </si>
   <si>
     <t>Onovo</t>
-  </si>
-  <si>
-    <t>TwentyFiveMayFiveB</t>
   </si>
 </sst>
 </file>
@@ -1723,7 +1730,7 @@
         <v>104</v>
       </c>
       <c r="AT2" s="18">
-        <v>9361115379</v>
+        <v>9361114444</v>
       </c>
       <c r="AU2" s="13" t="s">
         <v>105</v>
@@ -1738,7 +1745,7 @@
         <v>107</v>
       </c>
       <c r="AY2" s="19">
-        <v>141992998</v>
+        <v>141573040</v>
       </c>
       <c r="AZ2" s="13" t="s">
         <v>105</v>
@@ -1829,20 +1836,20 @@
       <c r="A3" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="B3" s="9">
-        <v>10698114</v>
+      <c r="B3" s="9" t="s">
+        <v>127</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>77</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E3" s="11" t="s">
         <v>79</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G3" s="12" t="s">
         <v>81</v>
@@ -1903,13 +1910,13 @@
         <v>91</v>
       </c>
       <c r="Z3" s="12" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="AA3" s="8" t="s">
         <v>93</v>
       </c>
       <c r="AB3" s="8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AC3" s="8" t="s">
         <v>95</v>
@@ -1948,10 +1955,10 @@
         <v>45597</v>
       </c>
       <c r="AN3" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AO3" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="AP3" s="11">
         <v>100</v>
@@ -1967,7 +1974,7 @@
         <v>104</v>
       </c>
       <c r="AT3" s="18">
-        <v>9361114774</v>
+        <v>9361113872</v>
       </c>
       <c r="AU3" s="13" t="s">
         <v>105</v>
@@ -1982,7 +1989,7 @@
         <v>107</v>
       </c>
       <c r="AY3" s="19">
-        <v>141982999</v>
+        <v>141563041</v>
       </c>
       <c r="AZ3" s="13" t="s">
         <v>105</v>
@@ -2051,10 +2058,10 @@
         <v>79</v>
       </c>
       <c r="BV3" s="20" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="BW3" s="20" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="BX3" s="20">
         <v>201</v>
@@ -2071,10 +2078,10 @@
     </row>
     <row r="4" spans="1:92" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>77</v>
@@ -2086,7 +2093,7 @@
         <v>79</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G4" s="12" t="s">
         <v>81</v>
@@ -2150,13 +2157,13 @@
         <v>92</v>
       </c>
       <c r="AA4" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AB4" s="8" t="s">
         <v>94</v>
       </c>
       <c r="AC4" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AD4" s="11" t="s">
         <v>96</v>
@@ -2165,7 +2172,7 @@
         <v>97</v>
       </c>
       <c r="AF4" s="8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="AG4" s="16">
         <v>20</v>
@@ -2196,7 +2203,7 @@
         <v>102</v>
       </c>
       <c r="AO4" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="AP4" s="11">
         <v>100</v>
@@ -2212,7 +2219,7 @@
         <v>104</v>
       </c>
       <c r="AT4" s="18">
-        <v>9361116116</v>
+        <v>9361114840</v>
       </c>
       <c r="AU4" s="13" t="s">
         <v>105</v>
@@ -2227,7 +2234,7 @@
         <v>107</v>
       </c>
       <c r="AY4" s="19">
-        <v>141973000</v>
+        <v>141703027</v>
       </c>
       <c r="AZ4" s="13" t="s">
         <v>105</v>
@@ -2266,10 +2273,10 @@
         <v>79</v>
       </c>
       <c r="BL4" s="14" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="BM4" s="14" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="BN4" s="14" t="s">
         <v>117</v>
@@ -2287,7 +2294,7 @@
         <v>1991</v>
       </c>
       <c r="BS4" s="14" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="BT4" s="14" t="s">
         <v>120</v>
@@ -2296,10 +2303,10 @@
         <v>79</v>
       </c>
       <c r="BV4" s="20" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="BW4" s="20" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="BX4" s="20">
         <v>213</v>
@@ -2316,22 +2323,22 @@
     </row>
     <row r="5" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="B5" s="9">
-        <v>10698116</v>
+        <v>148</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>149</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>77</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E5" s="11" t="s">
         <v>79</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="G5" s="12" t="s">
         <v>81</v>
@@ -2392,13 +2399,13 @@
         <v>91</v>
       </c>
       <c r="Z5" s="12" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="AA5" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AB5" s="8" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="AC5" s="8" t="s">
         <v>95</v>
@@ -2438,10 +2445,10 @@
         <v>45597</v>
       </c>
       <c r="AN5" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AO5" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="AP5" s="11">
         <v>100</v>
@@ -2457,7 +2464,7 @@
         <v>104</v>
       </c>
       <c r="AT5" s="18">
-        <v>9361111947</v>
+        <v>9361118448</v>
       </c>
       <c r="AU5" s="13" t="s">
         <v>105</v>
@@ -2472,7 +2479,7 @@
         <v>107</v>
       </c>
       <c r="AY5" s="19">
-        <v>141963001</v>
+        <v>141693028</v>
       </c>
       <c r="AZ5" s="13" t="s">
         <v>105</v>
@@ -2511,10 +2518,10 @@
         <v>79</v>
       </c>
       <c r="BL5" s="14" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="BM5" s="14" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="BN5" s="14" t="s">
         <v>117</v>
@@ -2532,7 +2539,7 @@
         <v>2024</v>
       </c>
       <c r="BS5" s="14" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="BT5" s="14" t="s">
         <v>120</v>
@@ -2541,10 +2548,10 @@
         <v>79</v>
       </c>
       <c r="BV5" s="20" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BW5" s="20" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BX5" s="20">
         <v>207</v>
@@ -2561,13 +2568,13 @@
     </row>
     <row r="6" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>78</v>
@@ -2576,7 +2583,7 @@
         <v>79</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="G6" s="12" t="s">
         <v>81</v>
@@ -2640,22 +2647,22 @@
         <v>92</v>
       </c>
       <c r="AA6" s="8" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="AB6" s="8" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="AC6" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AD6" s="11" t="s">
         <v>96</v>
       </c>
       <c r="AE6" s="11" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="AF6" s="8" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="AG6" s="16">
         <v>16</v>
@@ -2665,7 +2672,7 @@
         <v>45962</v>
       </c>
       <c r="AI6" s="12" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="AJ6" s="12" t="s">
         <v>101</v>
@@ -2686,7 +2693,7 @@
         <v>102</v>
       </c>
       <c r="AO6" s="8" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="AP6" s="11">
         <v>100</v>
@@ -2702,7 +2709,7 @@
         <v>104</v>
       </c>
       <c r="AT6" s="18">
-        <v>9361114928</v>
+        <v>9361118525</v>
       </c>
       <c r="AU6" s="13" t="s">
         <v>105</v>
@@ -2717,7 +2724,7 @@
         <v>107</v>
       </c>
       <c r="AY6" s="19">
-        <v>141953002</v>
+        <v>141683029</v>
       </c>
       <c r="AZ6" s="13" t="s">
         <v>105</v>
@@ -2786,10 +2793,10 @@
         <v>79</v>
       </c>
       <c r="BV6" s="20" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="BW6" s="20" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="BX6" s="20">
         <v>211</v>
@@ -2804,30 +2811,30 @@
         <v>125</v>
       </c>
     </row>
-    <row r="7" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E7" s="11" t="s">
         <v>79</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="G7" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H7" s="12" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="I7" s="12" t="s">
         <v>83</v>
@@ -2882,16 +2889,16 @@
         <v>91</v>
       </c>
       <c r="Z7" s="12" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="AA7" s="8" t="s">
         <v>93</v>
       </c>
       <c r="AB7" s="8" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="AC7" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AD7" s="11" t="s">
         <v>96</v>
@@ -2927,10 +2934,10 @@
         <v>45597</v>
       </c>
       <c r="AN7" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AO7" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="AP7" s="11">
         <v>100</v>
@@ -2946,7 +2953,7 @@
         <v>104</v>
       </c>
       <c r="AT7" s="18">
-        <v>9361115577</v>
+        <v>9361114037</v>
       </c>
       <c r="AU7" s="13" t="s">
         <v>105</v>
@@ -2961,7 +2968,7 @@
         <v>107</v>
       </c>
       <c r="AY7" s="19">
-        <v>141943003</v>
+        <v>141673030</v>
       </c>
       <c r="AZ7" s="13" t="s">
         <v>105</v>
@@ -3000,10 +3007,10 @@
         <v>79</v>
       </c>
       <c r="BL7" s="14" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="BM7" s="14" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="BN7" s="14" t="s">
         <v>117</v>
@@ -3021,7 +3028,7 @@
         <v>2000</v>
       </c>
       <c r="BS7" s="14" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="BT7" s="14" t="s">
         <v>120</v>
@@ -3030,10 +3037,10 @@
         <v>79</v>
       </c>
       <c r="BV7" s="20" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="BW7" s="20" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="BX7" s="20">
         <v>211</v>
@@ -3048,15 +3055,15 @@
         <v>125</v>
       </c>
     </row>
-    <row r="8" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>78</v>
@@ -3065,13 +3072,13 @@
         <v>79</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>244</v>
+        <v>81</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="I8" s="12" t="s">
         <v>83</v>
@@ -3129,13 +3136,13 @@
         <v>92</v>
       </c>
       <c r="AA8" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AB8" s="8" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="AC8" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AD8" s="11" t="s">
         <v>96</v>
@@ -3175,7 +3182,7 @@
         <v>102</v>
       </c>
       <c r="AO8" s="8" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="AP8" s="11">
         <v>100</v>
@@ -3191,7 +3198,7 @@
         <v>104</v>
       </c>
       <c r="AT8" s="18">
-        <v>9361114752</v>
+        <v>9361117931</v>
       </c>
       <c r="AU8" s="13" t="s">
         <v>105</v>
@@ -3206,7 +3213,7 @@
         <v>107</v>
       </c>
       <c r="AY8" s="19">
-        <v>141933004</v>
+        <v>141663031</v>
       </c>
       <c r="AZ8" s="13" t="s">
         <v>105</v>
@@ -3275,10 +3282,10 @@
         <v>79</v>
       </c>
       <c r="BV8" s="20" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="BW8" s="20" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="BX8" s="20">
         <v>213</v>
@@ -3295,28 +3302,28 @@
     </row>
     <row r="9" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>188</v>
-      </c>
-      <c r="B9" s="9">
-        <v>10698117</v>
+        <v>189</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>190</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>77</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E9" s="11" t="s">
         <v>79</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="G9" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="I9" s="12" t="s">
         <v>83</v>
@@ -3371,13 +3378,13 @@
         <v>91</v>
       </c>
       <c r="Z9" s="12" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="AA9" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AB9" s="8" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="AC9" s="8" t="s">
         <v>95</v>
@@ -3417,10 +3424,10 @@
         <v>45597</v>
       </c>
       <c r="AN9" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AO9" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="AP9" s="11">
         <v>100</v>
@@ -3436,7 +3443,7 @@
         <v>104</v>
       </c>
       <c r="AT9" s="18">
-        <v>9361112541</v>
+        <v>9361118415</v>
       </c>
       <c r="AU9" s="13" t="s">
         <v>105</v>
@@ -3451,7 +3458,7 @@
         <v>107</v>
       </c>
       <c r="AY9" s="19">
-        <v>141923005</v>
+        <v>141653032</v>
       </c>
       <c r="AZ9" s="13" t="s">
         <v>105</v>
@@ -3490,10 +3497,10 @@
         <v>79</v>
       </c>
       <c r="BL9" s="14" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="BM9" s="14" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="BN9" s="14" t="s">
         <v>117</v>
@@ -3511,7 +3518,7 @@
         <v>1991</v>
       </c>
       <c r="BS9" s="14" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="BT9" s="14" t="s">
         <v>120</v>
@@ -3520,10 +3527,10 @@
         <v>79</v>
       </c>
       <c r="BV9" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="BW9" s="20" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="BX9" s="20">
         <v>211</v>
@@ -3540,10 +3547,10 @@
     </row>
     <row r="10" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C10" s="8" t="s">
         <v>77</v>
@@ -3555,13 +3562,13 @@
         <v>79</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>182</v>
+        <v>81</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I10" s="12" t="s">
         <v>83</v>
@@ -3622,10 +3629,10 @@
         <v>93</v>
       </c>
       <c r="AB10" s="8" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="AC10" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AD10" s="11" t="s">
         <v>96</v>
@@ -3634,7 +3641,7 @@
         <v>97</v>
       </c>
       <c r="AF10" s="8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="AG10" s="16">
         <v>20</v>
@@ -3664,7 +3671,7 @@
         <v>102</v>
       </c>
       <c r="AO10" s="8" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="AP10" s="11">
         <v>100</v>
@@ -3680,7 +3687,7 @@
         <v>104</v>
       </c>
       <c r="AT10" s="18">
-        <v>9361113399</v>
+        <v>9361119724</v>
       </c>
       <c r="AU10" s="13" t="s">
         <v>105</v>
@@ -3695,7 +3702,7 @@
         <v>107</v>
       </c>
       <c r="AY10" s="19">
-        <v>141913006</v>
+        <v>141643033</v>
       </c>
       <c r="AZ10" s="13" t="s">
         <v>105</v>
@@ -3734,10 +3741,10 @@
         <v>79</v>
       </c>
       <c r="BL10" s="14" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="BM10" s="14" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="BN10" s="14" t="s">
         <v>117</v>
@@ -3755,7 +3762,7 @@
         <v>2024</v>
       </c>
       <c r="BS10" s="14" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="BT10" s="14" t="s">
         <v>120</v>
@@ -3764,10 +3771,10 @@
         <v>79</v>
       </c>
       <c r="BV10" s="20" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="BW10" s="20" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="BX10" s="20">
         <v>213</v>
@@ -3784,28 +3791,28 @@
     </row>
     <row r="11" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>77</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E11" s="11" t="s">
         <v>79</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="G11" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H11" s="12" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="I11" s="12" t="s">
         <v>83</v>
@@ -3860,13 +3867,13 @@
         <v>91</v>
       </c>
       <c r="Z11" s="12" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="AA11" s="8" t="s">
         <v>93</v>
       </c>
       <c r="AB11" s="8" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="AC11" s="8" t="s">
         <v>95</v>
@@ -3905,10 +3912,10 @@
         <v>45597</v>
       </c>
       <c r="AN11" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AO11" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="AP11" s="11">
         <v>100</v>
@@ -3924,7 +3931,7 @@
         <v>104</v>
       </c>
       <c r="AT11" s="18">
-        <v>9361113927</v>
+        <v>9361114532</v>
       </c>
       <c r="AU11" s="13" t="s">
         <v>105</v>
@@ -3939,7 +3946,7 @@
         <v>107</v>
       </c>
       <c r="AY11" s="19">
-        <v>141903007</v>
+        <v>141633034</v>
       </c>
       <c r="AZ11" s="13" t="s">
         <v>105</v>
@@ -4008,10 +4015,10 @@
         <v>79</v>
       </c>
       <c r="BV11" s="20" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="BW11" s="20" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="BX11" s="20">
         <v>201</v>
@@ -4028,10 +4035,10 @@
     </row>
     <row r="12" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>77</v>
@@ -4043,13 +4050,13 @@
         <v>79</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="G12" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H12" s="12" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="I12" s="12" t="s">
         <v>83</v>
@@ -4107,13 +4114,13 @@
         <v>92</v>
       </c>
       <c r="AA12" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AB12" s="8" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="AC12" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AD12" s="11" t="s">
         <v>96</v>
@@ -4153,7 +4160,7 @@
         <v>102</v>
       </c>
       <c r="AO12" s="8" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="AP12" s="11">
         <v>100</v>
@@ -4169,7 +4176,7 @@
         <v>104</v>
       </c>
       <c r="AT12" s="18">
-        <v>9361111078</v>
+        <v>9361114983</v>
       </c>
       <c r="AU12" s="13" t="s">
         <v>105</v>
@@ -4184,7 +4191,7 @@
         <v>107</v>
       </c>
       <c r="AY12" s="19">
-        <v>141893008</v>
+        <v>141623035</v>
       </c>
       <c r="AZ12" s="13" t="s">
         <v>105</v>
@@ -4223,10 +4230,10 @@
         <v>79</v>
       </c>
       <c r="BL12" s="14" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="BM12" s="14" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="BN12" s="14" t="s">
         <v>117</v>
@@ -4244,7 +4251,7 @@
         <v>2000</v>
       </c>
       <c r="BS12" s="14" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="BT12" s="14" t="s">
         <v>120</v>
@@ -4253,10 +4260,10 @@
         <v>79</v>
       </c>
       <c r="BV12" s="20" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="BW12" s="20" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="BX12" s="20">
         <v>213</v>
@@ -4273,28 +4280,28 @@
     </row>
     <row r="13" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>218</v>
-      </c>
-      <c r="B13" s="9">
-        <v>10698122</v>
+        <v>220</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>221</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>77</v>
+        <v>160</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E13" s="11" t="s">
         <v>79</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="G13" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H13" s="12" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="I13" s="12" t="s">
         <v>83</v>
@@ -4349,13 +4356,13 @@
         <v>91</v>
       </c>
       <c r="Z13" s="12" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="AA13" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AB13" s="8" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="AC13" s="8" t="s">
         <v>95</v>
@@ -4395,10 +4402,10 @@
         <v>45597</v>
       </c>
       <c r="AN13" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AO13" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="AP13" s="11">
         <v>100</v>
@@ -4414,7 +4421,7 @@
         <v>104</v>
       </c>
       <c r="AT13" s="18">
-        <v>9361113476</v>
+        <v>9361114774</v>
       </c>
       <c r="AU13" s="13" t="s">
         <v>105</v>
@@ -4429,7 +4436,7 @@
         <v>107</v>
       </c>
       <c r="AY13" s="19">
-        <v>141883009</v>
+        <v>141613036</v>
       </c>
       <c r="AZ13" s="13" t="s">
         <v>105</v>
@@ -4498,10 +4505,10 @@
         <v>79</v>
       </c>
       <c r="BV13" s="20" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="BW13" s="20" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="BX13" s="20">
         <v>209</v>
@@ -4518,10 +4525,10 @@
     </row>
     <row r="14" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>77</v>
@@ -4533,13 +4540,13 @@
         <v>79</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="G14" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H14" s="12" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="I14" s="12" t="s">
         <v>83</v>
@@ -4600,10 +4607,10 @@
         <v>93</v>
       </c>
       <c r="AB14" s="8" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="AC14" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AD14" s="11" t="s">
         <v>96</v>
@@ -4612,7 +4619,7 @@
         <v>97</v>
       </c>
       <c r="AF14" s="8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="AG14" s="16">
         <v>24</v>
@@ -4642,7 +4649,7 @@
         <v>102</v>
       </c>
       <c r="AO14" s="8" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="AP14" s="11">
         <v>100</v>
@@ -4658,7 +4665,7 @@
         <v>104</v>
       </c>
       <c r="AT14" s="18">
-        <v>9361115423</v>
+        <v>9361115060</v>
       </c>
       <c r="AU14" s="13" t="s">
         <v>105</v>
@@ -4673,7 +4680,7 @@
         <v>107</v>
       </c>
       <c r="AY14" s="19">
-        <v>141873010</v>
+        <v>141603037</v>
       </c>
       <c r="AZ14" s="13" t="s">
         <v>105</v>
@@ -4712,10 +4719,10 @@
         <v>79</v>
       </c>
       <c r="BL14" s="14" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="BM14" s="14" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="BN14" s="14" t="s">
         <v>117</v>
@@ -4733,7 +4740,7 @@
         <v>1991</v>
       </c>
       <c r="BS14" s="14" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="BT14" s="14" t="s">
         <v>120</v>
@@ -4742,10 +4749,10 @@
         <v>79</v>
       </c>
       <c r="BV14" s="20" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="BW14" s="20" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="BX14" s="20">
         <v>211</v>
@@ -4762,10 +4769,10 @@
     </row>
     <row r="15" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>77</v>
@@ -4777,13 +4784,13 @@
         <v>79</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="G15" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H15" s="12" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="I15" s="12" t="s">
         <v>83</v>
@@ -4841,10 +4848,10 @@
         <v>92</v>
       </c>
       <c r="AA15" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AB15" s="8" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="AC15" s="8" t="s">
         <v>95</v>
@@ -4887,7 +4894,7 @@
         <v>102</v>
       </c>
       <c r="AO15" s="8" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="AP15" s="11">
         <v>100</v>
@@ -4903,7 +4910,7 @@
         <v>104</v>
       </c>
       <c r="AT15" s="18">
-        <v>9361112728</v>
+        <v>9361113630</v>
       </c>
       <c r="AU15" s="13" t="s">
         <v>105</v>
@@ -4918,7 +4925,7 @@
         <v>107</v>
       </c>
       <c r="AY15" s="19">
-        <v>141863011</v>
+        <v>141593038</v>
       </c>
       <c r="AZ15" s="13" t="s">
         <v>105</v>
@@ -4957,10 +4964,10 @@
         <v>79</v>
       </c>
       <c r="BL15" s="14" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="BM15" s="14" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="BN15" s="14" t="s">
         <v>117</v>
@@ -4978,7 +4985,7 @@
         <v>2024</v>
       </c>
       <c r="BS15" s="14" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="BT15" s="14" t="s">
         <v>120</v>
@@ -4987,10 +4994,10 @@
         <v>79</v>
       </c>
       <c r="BV15" s="20" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="BW15" s="20" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="BX15" s="20">
         <v>213</v>
@@ -5007,10 +5014,10 @@
     </row>
     <row r="16" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="C16" s="8" t="s">
         <v>77</v>
@@ -5022,13 +5029,13 @@
         <v>79</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="G16" s="12" t="s">
         <v>81</v>
       </c>
       <c r="H16" s="12" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="I16" s="12" t="s">
         <v>83</v>
@@ -5092,7 +5099,7 @@
         <v>94</v>
       </c>
       <c r="AC16" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AD16" s="11" t="s">
         <v>96</v>
@@ -5131,7 +5138,7 @@
         <v>102</v>
       </c>
       <c r="AO16" s="8" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="AP16" s="11">
         <v>100</v>
@@ -5147,7 +5154,7 @@
         <v>104</v>
       </c>
       <c r="AT16" s="18">
-        <v>9361115896</v>
+        <v>9361113377</v>
       </c>
       <c r="AU16" s="13" t="s">
         <v>105</v>
@@ -5162,7 +5169,7 @@
         <v>107</v>
       </c>
       <c r="AY16" s="19">
-        <v>141853012</v>
+        <v>141583039</v>
       </c>
       <c r="AZ16" s="13" t="s">
         <v>105</v>
@@ -5201,10 +5208,10 @@
         <v>79</v>
       </c>
       <c r="BL16" s="14" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="BM16" s="14" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="BN16" s="14" t="s">
         <v>117</v>
@@ -5222,7 +5229,7 @@
         <v>2024</v>
       </c>
       <c r="BS16" s="14" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="BT16" s="14" t="s">
         <v>120</v>
@@ -5231,10 +5238,10 @@
         <v>79</v>
       </c>
       <c r="BV16" s="20" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="BW16" s="20" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="BX16" s="20">
         <v>211</v>

</xml_diff>